<commit_message>
Sprint 1: CSV support, security fixes, CLI polish, packaging
- Add CSV/TSV input support alongside Excel (.xlsx, .xls)
- Escape `why` text in HTML (_h) and PDF (_p) reports to prevent XSS/XML injection
- Fix blank_count/whitespace_only overlap — predicates now disjoint
- Switch HTML generation from string concat to list+join (O(n) vs O(n²))
- Pin dependency versions in requirements.txt
- Remove dead SEVERITY_COLORS dict
- Fix silent why-text fallback that used date explanation for all types
- Add input file type validation with clear error messages
- Add colored severity output (red/yellow/green) and per-sheet progress
- Add pyproject.toml with entry point (data-hygiene-audit CLI command)
- Update README with install instructions and CSV documentation
- Regenerate sample outputs with fixes applied
- Add full project audit (AUDIT.md) and improvement plan (PLAN.md)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/output/sample_messy_data_audit_findings.xlsx
+++ b/samples/output/sample_messy_data_audit_findings.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Findings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Findings'!$A$1:$H$60</definedName>
@@ -522,7 +522,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-04-27 13:40:28</t>
+          <t>2026-05-15 12:42:05</t>
         </is>
       </c>
     </row>
@@ -630,12 +630,12 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Mixed ID formats (some coded, some bare numbers)</t>
+          <t>Mixed ID formats</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>29 coded vs 1 bare numbers</t>
+          <t>29 coded (e.g. CUST-001) vs 1 bare numbers</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Null: 3, Blank: 1, Whitespace: 1</t>
+          <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Null: 3, Blank: 1, Whitespace: 1</t>
+          <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Null: 3, Blank: 1, Whitespace: 1</t>
+          <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Null: 3, Blank: 1, Whitespace: 1</t>
+          <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Null: 3, Blank: 1, Whitespace: 1</t>
+          <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Null: 3, Blank: 1, Whitespace: 1</t>
+          <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Null: 3, Blank: 1, Whitespace: 1</t>
+          <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>Null: 3, Blank: 1, Whitespace: 1</t>
+          <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Null: 14, Blank: 1, Whitespace: 1</t>
+          <t>Null: 14, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Vectorize detection.py for 3.4x speedup on large files
Replace Python-level per-element iteration with vectorized pandas
operations across all 6 hot functions: analyze_nulls, infer_field_type,
analyze_mixed_formats, analyze_wrong_purpose, analyze_phantom_duplicates,
and analyze_fuzzy_duplicates. 100K-row benchmark drops from 18.6s to 5.5s.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/output/sample_messy_data_audit_findings.xlsx
+++ b/samples/output/sample_messy_data_audit_findings.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Findings'!$A$1:$H$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Findings'!$A$1:$I$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +42,11 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -103,9 +108,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -488,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -505,35 +511,71 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>File:</t>
+          <t>Health Score:</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>sample_messy_data.xlsx</t>
+          <t>32/100</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Audit Date:</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-15 12:42:05</t>
+          <t>File:</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>sample_messy_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>Audit Date:</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:41:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>Total Issues:</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B6" s="4" t="n">
         <v>59</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Sheet: Customers</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Score: 0/100</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Sheet: Orders</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Score: 65/100</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -547,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -558,2530 +600,2926 @@
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="35" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Inferred Type</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Issue Type</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Example / Detail</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Why It Matters</t>
         </is>
       </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Suggested Fix</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>CustomerID</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Mixed ID formats</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>29 coded (e.g. CUST-001) vs 1 bare numbers</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>df["_CustomerID_format"] = df["CustomerID"].apply(
+    lambda x: "coded" if isinstance(x, str)
+    and "-" in x else "numeric"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>FirstName</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>df["FirstName"] = df["FirstName"].fillna(df["FirstName"].mode()[0])</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>FirstName</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Code/ID stuffed in name field</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>REF-4421</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t># Review rows where FirstName contains unexpected data
+mask = df["FirstName"].notna()
+suspect = df.loc[mask, "FirstName"]</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>FirstName</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Placeholder "Test" found 3 times</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>import numpy as np
+df["FirstName"] = df["FirstName"].replace("Test", np.nan)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>FirstName</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>import numpy as np
+df["FirstName"] = df["FirstName"].replace("TBD", np.nan)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>LastName</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>df["LastName"] = df["LastName"].fillna(df["LastName"].mode()[0])</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>LastName</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>import numpy as np
+df["LastName"] = df["LastName"].replace("TBD", np.nan)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>LastName</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>"User" repeated 3 times</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>df["_LastName_review"] = (
+    df["LastName"] == "User"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>LastName</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>"Doe" repeated 3 times</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>df["_LastName_review"] = (
+    df["LastName"] == "Doe"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>df["Email"] = df["Email"].fillna(df["Email"].mode()[0])</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Invalid email format</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>henrylee</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>email_re = r"^[a-zA-Z0-9._%+-]+@[a-zA-Z0-9.-]+\.[a-zA-Z]{2,}$"
+df["_Email_invalid"] = ~df["Email"].str.match(
+    email_re, na=False
+)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Invalid email format</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>nancy w@example.com</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>email_re = r"^[a-zA-Z0-9._%+-]+@[a-zA-Z0-9.-]+\.[a-zA-Z]{2,}$"
+df["_Email_invalid"] = ~df["Email"].str.match(
+    email_re, na=False
+)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>"test@test.com" repeated 3 times</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>df["_Email_review"] = (
+    df["Email"] == "test@test.com"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>df["Phone"] = df["Phone"].fillna(df["Phone"].mode()[0])</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Mixed phone formats: 17 values deviate from (XXX) XXX-XXXX</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>(XXX) XXX-XXXX: 9; XXX-XXX-XXXX: 8; (non-standard): 3; +1-XXX-XXX-XXXX: 2; XXXXXXXXXX: 1; XXX.XXX.XXXX: 1; XXX XXX XXXX: 1; (XXX)XXXXXXX: 1</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Inconsistent phone formats break deduplication, prevent reliable search/lookup, and cause issues with automated dialers or SMS systems. Two records for the same person may appear as different contacts if one says "(555) 123-4567" and another says "5551234567".</t>
         </is>
       </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>digits = df["Phone"].str.replace(r"\D", "", regex=True)
+digits = digits.str.slice(-10)
+df["Phone"] = (
+    "(" + digits.str[:3] + ") "
+    + digits.str[3:6] + "-" + digits.str[6:]
+)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>import numpy as np
+df["Phone"] = df["Phone"].replace("TBD", np.nan)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>"(555) 123-4567" repeated 3 times</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>df["_Phone_review"] = (
+    df["Phone"] == "(555) 123-4567"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>"000-000-0000" repeated 3 times</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>df["_Phone_review"] = (
+    df["Phone"] == "000-000-0000"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>"555-555-5555" repeated 3 times</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>df["_Phone_review"] = (
+    df["Phone"] == "555-555-5555"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>df["JoinDate"] = df["JoinDate"].fillna(df["JoinDate"].mode()[0])</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>Mixed date formats: 12 values deviate from YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>YYYY-MM-DD: 14; MM/DD/YYYY: 3; Mon DD, YYYY: 3; (non-standard): 1; YYYY/MM/DD: 1; M/D/YYYY: 1; DD-Mon-YYYY: 1; YYYY.MM.DD: 1; MM-DD-YYYY: 1</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>Mixed date formats cause sorting failures, broken filters, and incorrect calculations. A date stored as text ("Jan 15, 2023") won't sort chronologically next to "2023-01-15". Downstream tools, APIs, and reports will misparse or reject inconsistent dates.</t>
         </is>
       </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>df["JoinDate"] = pd.to_datetime(
+    df["JoinDate"], format="mixed", dayfirst=False
+).dt.strftime("%Y-%m-%d")</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>import numpy as np
+df["JoinDate"] = df["JoinDate"].replace("TBD", np.nan)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>"2023-01-01" repeated 6 times</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>23.1% of non-null values</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>df["_JoinDate_review"] = (
+    df["JoinDate"] == "2023-01-01"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>"2023-01-15" repeated 3 times</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>df["_JoinDate_review"] = (
+    df["JoinDate"] == "2023-01-15"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>df["AccountBalance"] = df["AccountBalance"].fillna(df["AccountBalance"].mode()[0])</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>Mixed currency formats: 11 values deviate from $X,XXX.XX</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>$X,XXX.XX: 15; X,XXX.XX (no symbol): 4; $X,XXX: 3; (non-standard): 2; $X,XXX.XX USD: 2</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>Mixed currency formats ("$1,250.00" vs "1250" vs "five thousand") prevent accurate aggregation and comparison. Summing a column with text-formatted currency returns errors or silently drops values, leading to wrong totals in financial reports.</t>
         </is>
       </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>df["AccountBalance"] = (
+    df["AccountBalance"].str.replace(r"[^\d.]", "", regex=True)
+    .astype(float)
+)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="E28" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>Text in currency field</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="H28" s="5" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>df["_AccountBalance_invalid"] = ~df["AccountBalance"].str.match(
+    r"^[\$\d,\.\-]+$", na=False
+)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>Text in currency field</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>five thousand</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>df["_AccountBalance_invalid"] = ~df["AccountBalance"].str.match(
+    r"^[\$\d,\.\-]+$", na=False
+)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr">
+      <c r="E30" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="G30" s="6" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H30" s="5" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>import numpy as np
+df["AccountBalance"] = df["AccountBalance"].replace("TBD", np.nan)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>"$0.00" repeated 6 times</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>23.1% of non-null values</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>df["_AccountBalance_review"] = (
+    df["AccountBalance"] == "$0.00"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E32" s="8" t="inlineStr">
+      <c r="E32" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>"$1,250.00" repeated 3 times</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H32" s="5" t="inlineStr">
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>df["_AccountBalance_review"] = (
+    df["AccountBalance"] == "$1,250.00"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
+      <c r="E33" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="G33" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr">
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>df["Status"] = df["Status"].fillna(df["Status"].mode()[0])</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="E34" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>Inconsistent casing in categorical values</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="G34" s="6" t="inlineStr">
         <is>
           <t>ACTIVE / Active / active</t>
         </is>
       </c>
-      <c r="H34" s="5" t="inlineStr">
+      <c r="H34" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t># Review rows where Status contains unexpected data
+mask = df["Status"].notna()
+suspect = df.loc[mask, "Status"]</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E35" s="7" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="G35" s="6" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H35" s="5" t="inlineStr">
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>import numpy as np
+df["Status"] = df["Status"].replace("TBD", np.nan)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="E36" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <t>"Active" repeated 18 times</t>
         </is>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="G36" s="6" t="inlineStr">
         <is>
           <t>69.2% of non-null values</t>
         </is>
       </c>
-      <c r="H36" s="5" t="inlineStr">
+      <c r="H36" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>df["_Status_review"] = (
+    df["Status"] == "Active"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="E37" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="G37" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H37" s="5" t="inlineStr">
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>df["ZipCode"] = df["ZipCode"].fillna(df["ZipCode"].mode()[0])</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E38" s="8" t="inlineStr">
+      <c r="E38" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F38" s="5" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>Placeholder "00000" found 3 times</t>
         </is>
       </c>
-      <c r="G38" s="5" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H38" s="5" t="inlineStr">
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>import numpy as np
+df["ZipCode"] = df["ZipCode"].replace("00000", np.nan)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E39" s="7" t="inlineStr">
+      <c r="E39" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="G39" s="6" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H39" s="5" t="inlineStr">
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>import numpy as np
+df["ZipCode"] = df["ZipCode"].replace("TBD", np.nan)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E40" s="8" t="inlineStr">
+      <c r="E40" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F40" s="5" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>"30301" repeated 3 times</t>
         </is>
       </c>
-      <c r="G40" s="5" t="inlineStr">
+      <c r="G40" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H40" s="5" t="inlineStr">
+      <c r="H40" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
+      <c r="I40" s="6" t="inlineStr">
+        <is>
+          <t>df["_ZipCode_review"] = (
+    df["ZipCode"] == "30301"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E41" s="8" t="inlineStr">
+      <c r="E41" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>"12345" repeated 3 times</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H41" s="5" t="inlineStr">
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>df["_ZipCode_review"] = (
+    df["ZipCode"] == "12345"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>freetext</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E42" s="8" t="inlineStr">
+      <c r="E42" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>15 of 30 values missing (50.0%)</t>
         </is>
       </c>
-      <c r="G42" s="5" t="inlineStr">
+      <c r="G42" s="6" t="inlineStr">
         <is>
           <t>Null: 14, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H42" s="5" t="inlineStr">
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t># Option A: Fill with most common value
+df["Notes"] = df["Notes"].fillna(df["Notes"].mode()[0])
+# Option B: Fill with a sentinel
+df["Notes"] = df["Notes"].fillna("MISSING")</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>freetext</t>
         </is>
       </c>
-      <c r="D43" s="5" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E43" s="8" t="inlineStr">
+      <c r="E43" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TEST" found 3 times</t>
         </is>
       </c>
-      <c r="G43" s="5" t="inlineStr">
+      <c r="G43" s="6" t="inlineStr">
         <is>
           <t>20.0% of non-null values</t>
         </is>
       </c>
-      <c r="H43" s="5" t="inlineStr">
+      <c r="H43" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
+      <c r="I43" s="6" t="inlineStr">
+        <is>
+          <t>import numpy as np
+df["Notes"] = df["Notes"].replace("TEST", np.nan)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="C44" s="6" t="inlineStr">
         <is>
           <t>freetext</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E44" s="8" t="inlineStr">
+      <c r="E44" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F44" s="5" t="inlineStr">
+      <c r="F44" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G44" s="5" t="inlineStr">
+      <c r="G44" s="6" t="inlineStr">
         <is>
           <t>6.7% of non-null values</t>
         </is>
       </c>
-      <c r="H44" s="5" t="inlineStr">
+      <c r="H44" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
+          <t>import numpy as np
+df["Notes"] = df["Notes"].replace("TBD", np.nan)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C45" s="5" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>freetext</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E45" s="8" t="inlineStr">
+      <c r="E45" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>"Preferred customer" repeated 3 times</t>
         </is>
       </c>
-      <c r="G45" s="5" t="inlineStr">
+      <c r="G45" s="6" t="inlineStr">
         <is>
           <t>20.0% of non-null values</t>
         </is>
       </c>
-      <c r="H45" s="5" t="inlineStr">
+      <c r="H45" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>df["_Notes_review"] = (
+    df["Notes"] == "Preferred customer"
+)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>Phantom Duplicate</t>
         </is>
       </c>
-      <c r="E46" s="8" t="inlineStr">
+      <c r="E46" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F46" s="5" t="inlineStr">
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <t>3 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr">
+      <c r="G46" s="6" t="inlineStr">
         <is>
           <t>Rows: 2, 8, 9</t>
         </is>
       </c>
-      <c r="H46" s="5" t="inlineStr">
+      <c r="H46" s="6" t="inlineStr">
         <is>
           <t>These records look different on the surface (different casing, extra spaces, punctuation variations) but represent the same entity. They cause inflated counts, split transaction histories, and duplicate outreach — problems that compound over time.</t>
         </is>
       </c>
+      <c r="I46" s="6" t="inlineStr">
+        <is>
+          <t># Normalize text columns before deduplication
+text_cols = df.select_dtypes(include="object").columns
+for col in text_cols:
+    df[col] = df[col].str.strip().str.lower()
+df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Phantom Duplicate</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr">
+      <c r="E47" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F47" s="5" t="inlineStr">
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <t>2 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr">
+      <c r="G47" s="6" t="inlineStr">
         <is>
           <t>Rows: 3, 10</t>
         </is>
       </c>
-      <c r="H47" s="5" t="inlineStr">
+      <c r="H47" s="6" t="inlineStr">
         <is>
           <t>These records look different on the surface (different casing, extra spaces, punctuation variations) but represent the same entity. They cause inflated counts, split transaction histories, and duplicate outreach — problems that compound over time.</t>
         </is>
       </c>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t># Normalize text columns before deduplication
+text_cols = df.select_dtypes(include="object").columns
+for col in text_cols:
+    df[col] = df[col].str.strip().str.lower()
+df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>Exact Duplicate</t>
         </is>
       </c>
-      <c r="E48" s="6" t="inlineStr">
+      <c r="E48" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F48" s="5" t="inlineStr">
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>3 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G48" s="5" t="inlineStr">
+      <c r="G48" s="6" t="inlineStr">
         <is>
           <t>Rows: 11, 12, 13</t>
         </is>
       </c>
-      <c r="H48" s="5" t="inlineStr">
+      <c r="H48" s="6" t="inlineStr">
         <is>
           <t>Exact duplicate rows are the clearest sign of a data quality issue — they can result from double-submissions, ETL failures, or missing unique constraints. Every duplicate inflates counts and distorts any metric built on this data.</t>
         </is>
       </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D49" s="5" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>Phantom Duplicate</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
+      <c r="E49" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>4 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G49" s="5" t="inlineStr">
+      <c r="G49" s="6" t="inlineStr">
         <is>
           <t>Rows: 14, 19, 20, 21</t>
         </is>
       </c>
-      <c r="H49" s="5" t="inlineStr">
+      <c r="H49" s="6" t="inlineStr">
         <is>
           <t>These records look different on the surface (different casing, extra spaces, punctuation variations) but represent the same entity. They cause inflated counts, split transaction histories, and duplicate outreach — problems that compound over time.</t>
         </is>
       </c>
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t># Normalize text columns before deduplication
+text_cols = df.select_dtypes(include="object").columns
+for col in text_cols:
+    df[col] = df[col].str.strip().str.lower()
+df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>Exact Duplicate</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="E50" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F50" s="5" t="inlineStr">
+      <c r="F50" s="6" t="inlineStr">
         <is>
           <t>2 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G50" s="5" t="inlineStr">
+      <c r="G50" s="6" t="inlineStr">
         <is>
           <t>Rows: 25, 27</t>
         </is>
       </c>
-      <c r="H50" s="5" t="inlineStr">
+      <c r="H50" s="6" t="inlineStr">
         <is>
           <t>Exact duplicate rows are the clearest sign of a data quality issue — they can result from double-submissions, ETL failures, or missing unique constraints. Every duplicate inflates counts and distorts any metric built on this data.</t>
         </is>
       </c>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B51" s="5" t="inlineStr">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>OrderDate</t>
         </is>
       </c>
-      <c r="C51" s="5" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D51" s="5" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="E51" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="F51" s="6" t="inlineStr">
         <is>
           <t>Mixed date formats: 4 values deviate from YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="G51" s="5" t="inlineStr">
+      <c r="G51" s="6" t="inlineStr">
         <is>
           <t>YYYY-MM-DD: 6; MM/DD/YYYY: 1; Mon DD, YYYY: 1; M/D/YYYY: 1; YYYY/MM/DD: 1</t>
         </is>
       </c>
-      <c r="H51" s="5" t="inlineStr">
+      <c r="H51" s="6" t="inlineStr">
         <is>
           <t>Mixed date formats cause sorting failures, broken filters, and incorrect calculations. A date stored as text ("Jan 15, 2023") won't sort chronologically next to "2023-01-15". Downstream tools, APIs, and reports will misparse or reject inconsistent dates.</t>
         </is>
       </c>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>df["OrderDate"] = pd.to_datetime(
+    df["OrderDate"], format="mixed", dayfirst=False
+).dt.strftime("%Y-%m-%d")</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B52" s="5" t="inlineStr">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E52" s="8" t="inlineStr">
+      <c r="E52" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <t>Mixed currency formats: 3 values deviate from $X,XXX.XX</t>
         </is>
       </c>
-      <c r="G52" s="5" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>$X,XXX.XX: 7; X,XXX (bare number): 2; $X,XXX: 1</t>
         </is>
       </c>
-      <c r="H52" s="5" t="inlineStr">
+      <c r="H52" s="6" t="inlineStr">
         <is>
           <t>Mixed currency formats ("$1,250.00" vs "1250" vs "five thousand") prevent accurate aggregation and comparison. Summing a column with text-formatted currency returns errors or silently drops values, leading to wrong totals in financial reports.</t>
         </is>
       </c>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>df["Amount"] = (
+    df["Amount"].str.replace(r"[^\d.]", "", regex=True)
+    .astype(float)
+)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B53" s="5" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>ShipDate</t>
         </is>
       </c>
-      <c r="C53" s="5" t="inlineStr">
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D53" s="5" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E53" s="7" t="inlineStr">
+      <c r="E53" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F53" s="5" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>2 of 10 values missing (20.0%)</t>
         </is>
       </c>
-      <c r="G53" s="5" t="inlineStr">
+      <c r="G53" s="6" t="inlineStr">
         <is>
           <t>Null: 2, Blank: 0, Whitespace: 0</t>
         </is>
       </c>
-      <c r="H53" s="5" t="inlineStr">
+      <c r="H53" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>df["ShipDate"] = df["ShipDate"].fillna(df["ShipDate"].mode()[0])</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B54" s="5" t="inlineStr">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>ShipDate</t>
         </is>
       </c>
-      <c r="C54" s="5" t="inlineStr">
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="E54" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F54" s="5" t="inlineStr">
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <t>Mixed date formats: 3 values deviate from YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="G54" s="5" t="inlineStr">
+      <c r="G54" s="6" t="inlineStr">
         <is>
           <t>YYYY-MM-DD: 5; MM/DD/YYYY: 1; Mon DD, YYYY: 1; M/D/YYYY: 1</t>
         </is>
       </c>
-      <c r="H54" s="5" t="inlineStr">
+      <c r="H54" s="6" t="inlineStr">
         <is>
           <t>Mixed date formats cause sorting failures, broken filters, and incorrect calculations. A date stored as text ("Jan 15, 2023") won't sort chronologically next to "2023-01-15". Downstream tools, APIs, and reports will misparse or reject inconsistent dates.</t>
         </is>
       </c>
+      <c r="I54" s="6" t="inlineStr">
+        <is>
+          <t>df["ShipDate"] = pd.to_datetime(
+    df["ShipDate"], format="mixed", dayfirst=False
+).dt.strftime("%Y-%m-%d")</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B55" s="5" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E55" s="6" t="inlineStr">
+      <c r="E55" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F55" s="5" t="inlineStr">
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>Inconsistent casing in categorical values</t>
         </is>
       </c>
-      <c r="G55" s="5" t="inlineStr">
+      <c r="G55" s="6" t="inlineStr">
         <is>
           <t>Shipped / shipped</t>
         </is>
       </c>
-      <c r="H55" s="5" t="inlineStr">
+      <c r="H55" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t># Review rows where Status contains unexpected data
+mask = df["Status"].notna()
+suspect = df.loc[mask, "Status"]</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B56" s="5" t="inlineStr">
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E56" s="6" t="inlineStr">
+      <c r="E56" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F56" s="5" t="inlineStr">
+      <c r="F56" s="6" t="inlineStr">
         <is>
           <t>Inconsistent casing in categorical values</t>
         </is>
       </c>
-      <c r="G56" s="5" t="inlineStr">
+      <c r="G56" s="6" t="inlineStr">
         <is>
           <t>Delivered / delivered</t>
         </is>
       </c>
-      <c r="H56" s="5" t="inlineStr">
+      <c r="H56" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t># Review rows where Status contains unexpected data
+mask = df["Status"].notna()
+suspect = df.loc[mask, "Status"]</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B57" s="5" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D57" s="5" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E57" s="6" t="inlineStr">
+      <c r="E57" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F57" s="5" t="inlineStr">
+      <c r="F57" s="6" t="inlineStr">
         <is>
           <t>Inconsistent casing in categorical values</t>
         </is>
       </c>
-      <c r="G57" s="5" t="inlineStr">
+      <c r="G57" s="6" t="inlineStr">
         <is>
           <t>PENDING / Pending</t>
         </is>
       </c>
-      <c r="H57" s="5" t="inlineStr">
+      <c r="H57" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
+      <c r="I57" s="6" t="inlineStr">
+        <is>
+          <t># Review rows where Status contains unexpected data
+mask = df["Status"].notna()
+suspect = df.loc[mask, "Status"]</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B58" s="5" t="inlineStr">
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E58" s="8" t="inlineStr">
+      <c r="E58" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F58" s="5" t="inlineStr">
+      <c r="F58" s="6" t="inlineStr">
         <is>
           <t>Placeholder "Test" found 2 times</t>
         </is>
       </c>
-      <c r="G58" s="5" t="inlineStr">
+      <c r="G58" s="6" t="inlineStr">
         <is>
           <t>20.0% of non-null values</t>
         </is>
       </c>
-      <c r="H58" s="5" t="inlineStr">
+      <c r="H58" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>import numpy as np
+df["Status"] = df["Status"].replace("Test", np.nan)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B59" s="5" t="inlineStr">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C59" s="5" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D59" s="5" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>Exact Duplicate</t>
         </is>
       </c>
-      <c r="E59" s="6" t="inlineStr">
+      <c r="E59" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F59" s="5" t="inlineStr">
+      <c r="F59" s="6" t="inlineStr">
         <is>
           <t>2 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G59" s="5" t="inlineStr">
+      <c r="G59" s="6" t="inlineStr">
         <is>
           <t>Rows: 5, 6</t>
         </is>
       </c>
-      <c r="H59" s="5" t="inlineStr">
+      <c r="H59" s="6" t="inlineStr">
         <is>
           <t>Exact duplicate rows are the clearest sign of a data quality issue — they can result from double-submissions, ETL failures, or missing unique constraints. Every duplicate inflates counts and distorts any metric built on this data.</t>
         </is>
       </c>
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+      <c r="A60" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B60" s="5" t="inlineStr">
+      <c r="B60" s="6" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C60" s="5" t="inlineStr">
+      <c r="C60" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
+      <c r="D60" s="6" t="inlineStr">
         <is>
           <t>Exact Duplicate</t>
         </is>
       </c>
-      <c r="E60" s="6" t="inlineStr">
+      <c r="E60" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F60" s="5" t="inlineStr">
+      <c r="F60" s="6" t="inlineStr">
         <is>
           <t>2 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G60" s="5" t="inlineStr">
+      <c r="G60" s="6" t="inlineStr">
         <is>
           <t>Rows: 7, 8</t>
         </is>
       </c>
-      <c r="H60" s="5" t="inlineStr">
+      <c r="H60" s="6" t="inlineStr">
         <is>
           <t>Exact duplicate rows are the clearest sign of a data quality issue — they can result from double-submissions, ETL failures, or missing unique constraints. Every duplicate inflates counts and distorts any metric built on this data.</t>
         </is>
       </c>
+      <c r="I60" s="6" t="inlineStr">
+        <is>
+          <t>df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H60"/>
+  <autoFilter ref="A1:I60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add schema validation and trend comparison features
Add --schema/-s flag for validating data against user-defined type
expectations (type mismatches, missing required columns, completeness
thresholds). Add --baseline/-b flag for comparing audits over time
with score and issue deltas. Add --generate-schema to bootstrap a
schema from inferred types. Includes 26 new tests, report integration
across HTML/Excel/PDF, and health score penalties for violations.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/output/sample_messy_data_audit_findings.xlsx
+++ b/samples/output/sample_messy_data_audit_findings.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -540,7 +540,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-15 14:41:31</t>
+          <t>2026-05-15 15:03:29</t>
         </is>
       </c>
     </row>
@@ -575,6 +575,49 @@
       <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Score: 65/100</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Trend vs Baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Baseline:</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>sample_messy_data.xlsx (2026-05-15 15:03:07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Score Change:</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>28 → 32 (+4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Issues Change:</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>63 → 59 (-4)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 5: CLI polish, counting fix, version/quiet flags, CHANGELOG
- Fix CLI issue count to include fuzzy duplicates and schema violations
  by extracting shared count_issues() helper used by CLI, HTML report
- Fix AuditResult._raw to be a proper dataclass field (type-safe)
- Remove _load_sheets from __all__ (internal, not public API)
- Add --version/-V, --quiet/-q, --force flags
- Add file size guard (warn 500K rows, refuse 2M without --force)
- Surface warning when Levenshtein matching is skipped (>500 rows)
- Raise minimum Python from 3.8 to 3.9 (pyproject + ruff + README)
- Add CHANGELOG.md (Keep a Changelog format)
- Document all CLI flags in README options table

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/output/sample_messy_data_audit_findings.xlsx
+++ b/samples/output/sample_messy_data_audit_findings.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -540,7 +540,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-15 15:03:29</t>
+          <t>2026-05-16 12:00:51</t>
         </is>
       </c>
     </row>
@@ -575,49 +575,6 @@
       <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Score: 65/100</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Trend vs Baseline</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Baseline:</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>sample_messy_data.xlsx (2026-05-15 15:03:07)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Score Change:</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>28 → 32 (+4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Issues Change:</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>63 → 59 (-4)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply Lailara design system branding to all report generators
Replace generic color palette with Lailara brand tokens (Chicago blue,
Hong Kong teal, Singapore orange, Red-42) across HTML, PDF, and Excel
reports. HTML gets Playfair Display + Source Sans 3 typography, warm
canvas background, and 2px border radius. PDF and Excel severity colors
and table headers updated to match.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/output/sample_messy_data_audit_findings.xlsx
+++ b/samples/output/sample_messy_data_audit_findings.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,28 +29,32 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Source Sans Pro"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Source Sans Pro"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Source Sans Pro"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Source Sans Pro"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Source Sans Pro"/>
+      <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -63,22 +67,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000f3460"/>
+        <fgColor rgb="001f2e7a"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
+        <fgColor rgb="00fce8e7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D4EDDA"/>
+        <fgColor rgb="00e4f5f0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
+        <fgColor rgb="00fdeee0"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,27 +96,28 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00cccccc"/>
+        <color rgb="00d9d9d9"/>
       </left>
       <right style="thin">
-        <color rgb="00cccccc"/>
+        <color rgb="00d9d9d9"/>
       </right>
       <top style="thin">
-        <color rgb="00cccccc"/>
+        <color rgb="00d9d9d9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00cccccc"/>
+        <color rgb="00d9d9d9"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -540,7 +545,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-16 12:00:51</t>
+          <t>2026-05-20 11:12:08</t>
         </is>
       </c>
     </row>
@@ -560,7 +565,7 @@
           <t>Sheet: Customers</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Score: 0/100</t>
         </is>
@@ -572,7 +577,7 @@
           <t>Sheet: Orders</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Score: 65/100</t>
         </is>
@@ -604,94 +609,94 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Inferred Type</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Issue Type</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Example / Detail</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Why It Matters</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Suggested Fix</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>CustomerID</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Mixed ID formats</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>29 coded (e.g. CUST-001) vs 1 bare numbers</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>df["_CustomerID_format"] = df["CustomerID"].apply(
     lambda x: "coded" if isinstance(x, str)
@@ -701,94 +706,94 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>FirstName</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>df["FirstName"] = df["FirstName"].fillna(df["FirstName"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>FirstName</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Code/ID stuffed in name field</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>REF-4421</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t># Review rows where FirstName contains unexpected data
 mask = df["FirstName"].notna()
@@ -797,47 +802,47 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>FirstName</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Placeholder "Test" found 3 times</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>import numpy as np
 df["FirstName"] = df["FirstName"].replace("Test", np.nan)</t>
@@ -845,47 +850,47 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>FirstName</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>import numpy as np
 df["FirstName"] = df["FirstName"].replace("TBD", np.nan)</t>
@@ -893,94 +898,94 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>LastName</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>df["LastName"] = df["LastName"].fillna(df["LastName"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>LastName</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I8" s="7" t="inlineStr">
         <is>
           <t>import numpy as np
 df["LastName"] = df["LastName"].replace("TBD", np.nan)</t>
@@ -988,47 +993,47 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>LastName</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>"User" repeated 3 times</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I9" s="7" t="inlineStr">
         <is>
           <t>df["_LastName_review"] = (
     df["LastName"] == "User"
@@ -1037,47 +1042,47 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>LastName</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>"Doe" repeated 3 times</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>df["_LastName_review"] = (
     df["LastName"] == "Doe"
@@ -1086,94 +1091,94 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I11" s="7" t="inlineStr">
         <is>
           <t>df["Email"] = df["Email"].fillna(df["Email"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>Invalid email format</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>henrylee</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="I12" s="7" t="inlineStr">
         <is>
           <t>email_re = r"^[a-zA-Z0-9._%+-]+@[a-zA-Z0-9.-]+\.[a-zA-Z]{2,}$"
 df["_Email_invalid"] = ~df["Email"].str.match(
@@ -1183,47 +1188,47 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>Invalid email format</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>nancy w@example.com</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="I13" s="7" t="inlineStr">
         <is>
           <t>email_re = r"^[a-zA-Z0-9._%+-]+@[a-zA-Z0-9.-]+\.[a-zA-Z]{2,}$"
 df["_Email_invalid"] = ~df["Email"].str.match(
@@ -1233,47 +1238,47 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>"test@test.com" repeated 3 times</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr">
+      <c r="I14" s="7" t="inlineStr">
         <is>
           <t>df["_Email_review"] = (
     df["Email"] == "test@test.com"
@@ -1282,94 +1287,94 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>df["Phone"] = df["Phone"].fillna(df["Phone"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>Mixed phone formats: 17 values deviate from (XXX) XXX-XXXX</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>(XXX) XXX-XXXX: 9; XXX-XXX-XXXX: 8; (non-standard): 3; +1-XXX-XXX-XXXX: 2; XXXXXXXXXX: 1; XXX.XXX.XXXX: 1; XXX XXX XXXX: 1; (XXX)XXXXXXX: 1</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>Inconsistent phone formats break deduplication, prevent reliable search/lookup, and cause issues with automated dialers or SMS systems. Two records for the same person may appear as different contacts if one says "(555) 123-4567" and another says "5551234567".</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="I16" s="7" t="inlineStr">
         <is>
           <t>digits = df["Phone"].str.replace(r"\D", "", regex=True)
 digits = digits.str.slice(-10)
@@ -1381,47 +1386,47 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="I17" s="7" t="inlineStr">
         <is>
           <t>import numpy as np
 df["Phone"] = df["Phone"].replace("TBD", np.nan)</t>
@@ -1429,47 +1434,47 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>"(555) 123-4567" repeated 3 times</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I18" s="6" t="inlineStr">
+      <c r="I18" s="7" t="inlineStr">
         <is>
           <t>df["_Phone_review"] = (
     df["Phone"] == "(555) 123-4567"
@@ -1478,47 +1483,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>"000-000-0000" repeated 3 times</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I19" s="7" t="inlineStr">
         <is>
           <t>df["_Phone_review"] = (
     df["Phone"] == "000-000-0000"
@@ -1527,47 +1532,47 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>"555-555-5555" repeated 3 times</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr">
+      <c r="I20" s="7" t="inlineStr">
         <is>
           <t>df["_Phone_review"] = (
     df["Phone"] == "555-555-5555"
@@ -1576,94 +1581,94 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I21" s="6" t="inlineStr">
+      <c r="I21" s="7" t="inlineStr">
         <is>
           <t>df["JoinDate"] = df["JoinDate"].fillna(df["JoinDate"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>Mixed date formats: 12 values deviate from YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>YYYY-MM-DD: 14; MM/DD/YYYY: 3; Mon DD, YYYY: 3; (non-standard): 1; YYYY/MM/DD: 1; M/D/YYYY: 1; DD-Mon-YYYY: 1; YYYY.MM.DD: 1; MM-DD-YYYY: 1</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr">
         <is>
           <t>Mixed date formats cause sorting failures, broken filters, and incorrect calculations. A date stored as text ("Jan 15, 2023") won't sort chronologically next to "2023-01-15". Downstream tools, APIs, and reports will misparse or reject inconsistent dates.</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr">
+      <c r="I22" s="7" t="inlineStr">
         <is>
           <t>df["JoinDate"] = pd.to_datetime(
     df["JoinDate"], format="mixed", dayfirst=False
@@ -1672,47 +1677,47 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I23" s="6" t="inlineStr">
+      <c r="I23" s="7" t="inlineStr">
         <is>
           <t>import numpy as np
 df["JoinDate"] = df["JoinDate"].replace("TBD", np.nan)</t>
@@ -1720,47 +1725,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>"2023-01-01" repeated 6 times</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>23.1% of non-null values</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="H24" s="7" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr">
+      <c r="I24" s="7" t="inlineStr">
         <is>
           <t>df["_JoinDate_review"] = (
     df["JoinDate"] == "2023-01-01"
@@ -1769,47 +1774,47 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>"2023-01-15" repeated 3 times</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="H25" s="7" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr">
+      <c r="I25" s="7" t="inlineStr">
         <is>
           <t>df["_JoinDate_review"] = (
     df["JoinDate"] == "2023-01-15"
@@ -1818,94 +1823,94 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="F26" s="7" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="H26" s="7" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr">
+      <c r="I26" s="7" t="inlineStr">
         <is>
           <t>df["AccountBalance"] = df["AccountBalance"].fillna(df["AccountBalance"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Mixed currency formats: 11 values deviate from $X,XXX.XX</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>$X,XXX.XX: 15; X,XXX.XX (no symbol): 4; $X,XXX: 3; (non-standard): 2; $X,XXX.XX USD: 2</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="H27" s="7" t="inlineStr">
         <is>
           <t>Mixed currency formats ("$1,250.00" vs "1250" vs "five thousand") prevent accurate aggregation and comparison. Summing a column with text-formatted currency returns errors or silently drops values, leading to wrong totals in financial reports.</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr">
+      <c r="I27" s="7" t="inlineStr">
         <is>
           <t>df["AccountBalance"] = (
     df["AccountBalance"].str.replace(r"[^\d.]", "", regex=True)
@@ -1915,47 +1920,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E28" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="F28" s="7" t="inlineStr">
         <is>
           <t>Text in currency field</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="G28" s="7" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="H28" s="7" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr">
+      <c r="I28" s="7" t="inlineStr">
         <is>
           <t>df["_AccountBalance_invalid"] = ~df["AccountBalance"].str.match(
     r"^[\$\d,\.\-]+$", na=False
@@ -1964,47 +1969,47 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>Text in currency field</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>five thousand</t>
         </is>
       </c>
-      <c r="H29" s="6" t="inlineStr">
+      <c r="H29" s="7" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I29" s="6" t="inlineStr">
+      <c r="I29" s="7" t="inlineStr">
         <is>
           <t>df["_AccountBalance_invalid"] = ~df["AccountBalance"].str.match(
     r"^[\$\d,\.\-]+$", na=False
@@ -2013,47 +2018,47 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E30" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="F30" s="7" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="G30" s="7" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="H30" s="7" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I30" s="6" t="inlineStr">
+      <c r="I30" s="7" t="inlineStr">
         <is>
           <t>import numpy as np
 df["AccountBalance"] = df["AccountBalance"].replace("TBD", np.nan)</t>
@@ -2061,47 +2066,47 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="F31" s="7" t="inlineStr">
         <is>
           <t>"$0.00" repeated 6 times</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>23.1% of non-null values</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="H31" s="7" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I31" s="6" t="inlineStr">
+      <c r="I31" s="7" t="inlineStr">
         <is>
           <t>df["_AccountBalance_review"] = (
     df["AccountBalance"] == "$0.00"
@@ -2110,47 +2115,47 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E32" s="9" t="inlineStr">
+      <c r="E32" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>"$1,250.00" repeated 3 times</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
+      <c r="G32" s="7" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="H32" s="7" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I32" s="6" t="inlineStr">
+      <c r="I32" s="7" t="inlineStr">
         <is>
           <t>df["_AccountBalance_review"] = (
     df["AccountBalance"] == "$1,250.00"
@@ -2159,94 +2164,94 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr">
+      <c r="E33" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F33" s="6" t="inlineStr">
+      <c r="F33" s="7" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="G33" s="7" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="H33" s="7" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I33" s="6" t="inlineStr">
+      <c r="I33" s="7" t="inlineStr">
         <is>
           <t>df["Status"] = df["Status"].fillna(df["Status"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="F34" s="7" t="inlineStr">
         <is>
           <t>Inconsistent casing in categorical values</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr">
+      <c r="G34" s="7" t="inlineStr">
         <is>
           <t>ACTIVE / Active / active</t>
         </is>
       </c>
-      <c r="H34" s="6" t="inlineStr">
+      <c r="H34" s="7" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I34" s="6" t="inlineStr">
+      <c r="I34" s="7" t="inlineStr">
         <is>
           <t># Review rows where Status contains unexpected data
 mask = df["Status"].notna()
@@ -2255,47 +2260,47 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E35" s="8" t="inlineStr">
+      <c r="E35" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr">
+      <c r="F35" s="7" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G35" s="6" t="inlineStr">
+      <c r="G35" s="7" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H35" s="6" t="inlineStr">
+      <c r="H35" s="7" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I35" s="6" t="inlineStr">
+      <c r="I35" s="7" t="inlineStr">
         <is>
           <t>import numpy as np
 df["Status"] = df["Status"].replace("TBD", np.nan)</t>
@@ -2303,47 +2308,47 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C36" s="7" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D36" s="7" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="E36" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr">
+      <c r="F36" s="7" t="inlineStr">
         <is>
           <t>"Active" repeated 18 times</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr">
+      <c r="G36" s="7" t="inlineStr">
         <is>
           <t>69.2% of non-null values</t>
         </is>
       </c>
-      <c r="H36" s="6" t="inlineStr">
+      <c r="H36" s="7" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I36" s="6" t="inlineStr">
+      <c r="I36" s="7" t="inlineStr">
         <is>
           <t>df["_Status_review"] = (
     df["Status"] == "Active"
@@ -2352,94 +2357,94 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E37" s="8" t="inlineStr">
+      <c r="E37" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="G37" s="7" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr">
+      <c r="H37" s="7" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I37" s="6" t="inlineStr">
+      <c r="I37" s="7" t="inlineStr">
         <is>
           <t>df["ZipCode"] = df["ZipCode"].fillna(df["ZipCode"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D38" s="7" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E38" s="9" t="inlineStr">
+      <c r="E38" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F38" s="6" t="inlineStr">
+      <c r="F38" s="7" t="inlineStr">
         <is>
           <t>Placeholder "00000" found 3 times</t>
         </is>
       </c>
-      <c r="G38" s="6" t="inlineStr">
+      <c r="G38" s="7" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H38" s="6" t="inlineStr">
+      <c r="H38" s="7" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I38" s="6" t="inlineStr">
+      <c r="I38" s="7" t="inlineStr">
         <is>
           <t>import numpy as np
 df["ZipCode"] = df["ZipCode"].replace("00000", np.nan)</t>
@@ -2447,47 +2452,47 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E39" s="8" t="inlineStr">
+      <c r="E39" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr">
+      <c r="F39" s="7" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G39" s="6" t="inlineStr">
+      <c r="G39" s="7" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H39" s="6" t="inlineStr">
+      <c r="H39" s="7" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I39" s="6" t="inlineStr">
+      <c r="I39" s="7" t="inlineStr">
         <is>
           <t>import numpy as np
 df["ZipCode"] = df["ZipCode"].replace("TBD", np.nan)</t>
@@ -2495,47 +2500,47 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E40" s="9" t="inlineStr">
+      <c r="E40" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F40" s="6" t="inlineStr">
+      <c r="F40" s="7" t="inlineStr">
         <is>
           <t>"30301" repeated 3 times</t>
         </is>
       </c>
-      <c r="G40" s="6" t="inlineStr">
+      <c r="G40" s="7" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H40" s="6" t="inlineStr">
+      <c r="H40" s="7" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I40" s="6" t="inlineStr">
+      <c r="I40" s="7" t="inlineStr">
         <is>
           <t>df["_ZipCode_review"] = (
     df["ZipCode"] == "30301"
@@ -2544,47 +2549,47 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="D41" s="7" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E41" s="9" t="inlineStr">
+      <c r="E41" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F41" s="6" t="inlineStr">
+      <c r="F41" s="7" t="inlineStr">
         <is>
           <t>"12345" repeated 3 times</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr">
+      <c r="G41" s="7" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H41" s="6" t="inlineStr">
+      <c r="H41" s="7" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I41" s="6" t="inlineStr">
+      <c r="I41" s="7" t="inlineStr">
         <is>
           <t>df["_ZipCode_review"] = (
     df["ZipCode"] == "12345"
@@ -2593,47 +2598,47 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C42" s="7" t="inlineStr">
         <is>
           <t>freetext</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D42" s="7" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E42" s="9" t="inlineStr">
+      <c r="E42" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F42" s="6" t="inlineStr">
+      <c r="F42" s="7" t="inlineStr">
         <is>
           <t>15 of 30 values missing (50.0%)</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr">
+      <c r="G42" s="7" t="inlineStr">
         <is>
           <t>Null: 14, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H42" s="6" t="inlineStr">
+      <c r="H42" s="7" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I42" s="6" t="inlineStr">
+      <c r="I42" s="7" t="inlineStr">
         <is>
           <t># Option A: Fill with most common value
 df["Notes"] = df["Notes"].fillna(df["Notes"].mode()[0])
@@ -2643,47 +2648,47 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C43" s="6" t="inlineStr">
+      <c r="C43" s="7" t="inlineStr">
         <is>
           <t>freetext</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="D43" s="7" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E43" s="9" t="inlineStr">
+      <c r="E43" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F43" s="6" t="inlineStr">
+      <c r="F43" s="7" t="inlineStr">
         <is>
           <t>Placeholder "TEST" found 3 times</t>
         </is>
       </c>
-      <c r="G43" s="6" t="inlineStr">
+      <c r="G43" s="7" t="inlineStr">
         <is>
           <t>20.0% of non-null values</t>
         </is>
       </c>
-      <c r="H43" s="6" t="inlineStr">
+      <c r="H43" s="7" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I43" s="6" t="inlineStr">
+      <c r="I43" s="7" t="inlineStr">
         <is>
           <t>import numpy as np
 df["Notes"] = df["Notes"].replace("TEST", np.nan)</t>
@@ -2691,47 +2696,47 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C44" s="6" t="inlineStr">
+      <c r="C44" s="7" t="inlineStr">
         <is>
           <t>freetext</t>
         </is>
       </c>
-      <c r="D44" s="6" t="inlineStr">
+      <c r="D44" s="7" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E44" s="9" t="inlineStr">
+      <c r="E44" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F44" s="6" t="inlineStr">
+      <c r="F44" s="7" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G44" s="6" t="inlineStr">
+      <c r="G44" s="7" t="inlineStr">
         <is>
           <t>6.7% of non-null values</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr">
+      <c r="H44" s="7" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I44" s="6" t="inlineStr">
+      <c r="I44" s="7" t="inlineStr">
         <is>
           <t>import numpy as np
 df["Notes"] = df["Notes"].replace("TBD", np.nan)</t>
@@ -2739,47 +2744,47 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="inlineStr">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C45" s="7" t="inlineStr">
         <is>
           <t>freetext</t>
         </is>
       </c>
-      <c r="D45" s="6" t="inlineStr">
+      <c r="D45" s="7" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E45" s="9" t="inlineStr">
+      <c r="E45" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F45" s="6" t="inlineStr">
+      <c r="F45" s="7" t="inlineStr">
         <is>
           <t>"Preferred customer" repeated 3 times</t>
         </is>
       </c>
-      <c r="G45" s="6" t="inlineStr">
+      <c r="G45" s="7" t="inlineStr">
         <is>
           <t>20.0% of non-null values</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr">
+      <c r="H45" s="7" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I45" s="6" t="inlineStr">
+      <c r="I45" s="7" t="inlineStr">
         <is>
           <t>df["_Notes_review"] = (
     df["Notes"] == "Preferred customer"
@@ -2788,47 +2793,47 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C46" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D46" s="7" t="inlineStr">
         <is>
           <t>Phantom Duplicate</t>
         </is>
       </c>
-      <c r="E46" s="9" t="inlineStr">
+      <c r="E46" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F46" s="6" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>3 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G46" s="6" t="inlineStr">
+      <c r="G46" s="7" t="inlineStr">
         <is>
           <t>Rows: 2, 8, 9</t>
         </is>
       </c>
-      <c r="H46" s="6" t="inlineStr">
+      <c r="H46" s="7" t="inlineStr">
         <is>
           <t>These records look different on the surface (different casing, extra spaces, punctuation variations) but represent the same entity. They cause inflated counts, split transaction histories, and duplicate outreach — problems that compound over time.</t>
         </is>
       </c>
-      <c r="I46" s="6" t="inlineStr">
+      <c r="I46" s="7" t="inlineStr">
         <is>
           <t># Normalize text columns before deduplication
 text_cols = df.select_dtypes(include="object").columns
@@ -2839,47 +2844,47 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C47" s="6" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D47" s="6" t="inlineStr">
+      <c r="D47" s="7" t="inlineStr">
         <is>
           <t>Phantom Duplicate</t>
         </is>
       </c>
-      <c r="E47" s="9" t="inlineStr">
+      <c r="E47" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F47" s="6" t="inlineStr">
+      <c r="F47" s="7" t="inlineStr">
         <is>
           <t>2 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G47" s="6" t="inlineStr">
+      <c r="G47" s="7" t="inlineStr">
         <is>
           <t>Rows: 3, 10</t>
         </is>
       </c>
-      <c r="H47" s="6" t="inlineStr">
+      <c r="H47" s="7" t="inlineStr">
         <is>
           <t>These records look different on the surface (different casing, extra spaces, punctuation variations) but represent the same entity. They cause inflated counts, split transaction histories, and duplicate outreach — problems that compound over time.</t>
         </is>
       </c>
-      <c r="I47" s="6" t="inlineStr">
+      <c r="I47" s="7" t="inlineStr">
         <is>
           <t># Normalize text columns before deduplication
 text_cols = df.select_dtypes(include="object").columns
@@ -2890,94 +2895,94 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B48" s="6" t="inlineStr">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="C48" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="D48" s="7" t="inlineStr">
         <is>
           <t>Exact Duplicate</t>
         </is>
       </c>
-      <c r="E48" s="7" t="inlineStr">
+      <c r="E48" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F48" s="6" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
         <is>
           <t>3 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G48" s="6" t="inlineStr">
+      <c r="G48" s="7" t="inlineStr">
         <is>
           <t>Rows: 11, 12, 13</t>
         </is>
       </c>
-      <c r="H48" s="6" t="inlineStr">
+      <c r="H48" s="7" t="inlineStr">
         <is>
           <t>Exact duplicate rows are the clearest sign of a data quality issue — they can result from double-submissions, ETL failures, or missing unique constraints. Every duplicate inflates counts and distorts any metric built on this data.</t>
         </is>
       </c>
-      <c r="I48" s="6" t="inlineStr">
+      <c r="I48" s="7" t="inlineStr">
         <is>
           <t>df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="C49" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="D49" s="7" t="inlineStr">
         <is>
           <t>Phantom Duplicate</t>
         </is>
       </c>
-      <c r="E49" s="7" t="inlineStr">
+      <c r="E49" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F49" s="6" t="inlineStr">
+      <c r="F49" s="7" t="inlineStr">
         <is>
           <t>4 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G49" s="6" t="inlineStr">
+      <c r="G49" s="7" t="inlineStr">
         <is>
           <t>Rows: 14, 19, 20, 21</t>
         </is>
       </c>
-      <c r="H49" s="6" t="inlineStr">
+      <c r="H49" s="7" t="inlineStr">
         <is>
           <t>These records look different on the surface (different casing, extra spaces, punctuation variations) but represent the same entity. They cause inflated counts, split transaction histories, and duplicate outreach — problems that compound over time.</t>
         </is>
       </c>
-      <c r="I49" s="6" t="inlineStr">
+      <c r="I49" s="7" t="inlineStr">
         <is>
           <t># Normalize text columns before deduplication
 text_cols = df.select_dtypes(include="object").columns
@@ -2988,94 +2993,94 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C50" s="6" t="inlineStr">
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D50" s="6" t="inlineStr">
+      <c r="D50" s="7" t="inlineStr">
         <is>
           <t>Exact Duplicate</t>
         </is>
       </c>
-      <c r="E50" s="7" t="inlineStr">
+      <c r="E50" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F50" s="6" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
         <is>
           <t>2 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G50" s="6" t="inlineStr">
+      <c r="G50" s="7" t="inlineStr">
         <is>
           <t>Rows: 25, 27</t>
         </is>
       </c>
-      <c r="H50" s="6" t="inlineStr">
+      <c r="H50" s="7" t="inlineStr">
         <is>
           <t>Exact duplicate rows are the clearest sign of a data quality issue — they can result from double-submissions, ETL failures, or missing unique constraints. Every duplicate inflates counts and distorts any metric built on this data.</t>
         </is>
       </c>
-      <c r="I50" s="6" t="inlineStr">
+      <c r="I50" s="7" t="inlineStr">
         <is>
           <t>df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="inlineStr">
+      <c r="A51" s="7" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B51" s="7" t="inlineStr">
         <is>
           <t>OrderDate</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="C51" s="7" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D51" s="6" t="inlineStr">
+      <c r="D51" s="7" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E51" s="7" t="inlineStr">
+      <c r="E51" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F51" s="6" t="inlineStr">
+      <c r="F51" s="7" t="inlineStr">
         <is>
           <t>Mixed date formats: 4 values deviate from YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="G51" s="6" t="inlineStr">
+      <c r="G51" s="7" t="inlineStr">
         <is>
           <t>YYYY-MM-DD: 6; MM/DD/YYYY: 1; Mon DD, YYYY: 1; M/D/YYYY: 1; YYYY/MM/DD: 1</t>
         </is>
       </c>
-      <c r="H51" s="6" t="inlineStr">
+      <c r="H51" s="7" t="inlineStr">
         <is>
           <t>Mixed date formats cause sorting failures, broken filters, and incorrect calculations. A date stored as text ("Jan 15, 2023") won't sort chronologically next to "2023-01-15". Downstream tools, APIs, and reports will misparse or reject inconsistent dates.</t>
         </is>
       </c>
-      <c r="I51" s="6" t="inlineStr">
+      <c r="I51" s="7" t="inlineStr">
         <is>
           <t>df["OrderDate"] = pd.to_datetime(
     df["OrderDate"], format="mixed", dayfirst=False
@@ -3084,47 +3089,47 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="inlineStr">
+      <c r="A52" s="7" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B52" s="7" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr">
+      <c r="D52" s="7" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E52" s="9" t="inlineStr">
+      <c r="E52" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F52" s="6" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
         <is>
           <t>Mixed currency formats: 3 values deviate from $X,XXX.XX</t>
         </is>
       </c>
-      <c r="G52" s="6" t="inlineStr">
+      <c r="G52" s="7" t="inlineStr">
         <is>
           <t>$X,XXX.XX: 7; X,XXX (bare number): 2; $X,XXX: 1</t>
         </is>
       </c>
-      <c r="H52" s="6" t="inlineStr">
+      <c r="H52" s="7" t="inlineStr">
         <is>
           <t>Mixed currency formats ("$1,250.00" vs "1250" vs "five thousand") prevent accurate aggregation and comparison. Summing a column with text-formatted currency returns errors or silently drops values, leading to wrong totals in financial reports.</t>
         </is>
       </c>
-      <c r="I52" s="6" t="inlineStr">
+      <c r="I52" s="7" t="inlineStr">
         <is>
           <t>df["Amount"] = (
     df["Amount"].str.replace(r"[^\d.]", "", regex=True)
@@ -3134,94 +3139,94 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="inlineStr">
+      <c r="A53" s="7" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B53" s="7" t="inlineStr">
         <is>
           <t>ShipDate</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C53" s="7" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="D53" s="7" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E53" s="8" t="inlineStr">
+      <c r="E53" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
+      <c r="F53" s="7" t="inlineStr">
         <is>
           <t>2 of 10 values missing (20.0%)</t>
         </is>
       </c>
-      <c r="G53" s="6" t="inlineStr">
+      <c r="G53" s="7" t="inlineStr">
         <is>
           <t>Null: 2, Blank: 0, Whitespace: 0</t>
         </is>
       </c>
-      <c r="H53" s="6" t="inlineStr">
+      <c r="H53" s="7" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I53" s="6" t="inlineStr">
+      <c r="I53" s="7" t="inlineStr">
         <is>
           <t>df["ShipDate"] = df["ShipDate"].fillna(df["ShipDate"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+      <c r="A54" s="7" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B54" s="7" t="inlineStr">
         <is>
           <t>ShipDate</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C54" s="7" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr">
+      <c r="D54" s="7" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E54" s="7" t="inlineStr">
+      <c r="E54" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F54" s="6" t="inlineStr">
+      <c r="F54" s="7" t="inlineStr">
         <is>
           <t>Mixed date formats: 3 values deviate from YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="G54" s="6" t="inlineStr">
+      <c r="G54" s="7" t="inlineStr">
         <is>
           <t>YYYY-MM-DD: 5; MM/DD/YYYY: 1; Mon DD, YYYY: 1; M/D/YYYY: 1</t>
         </is>
       </c>
-      <c r="H54" s="6" t="inlineStr">
+      <c r="H54" s="7" t="inlineStr">
         <is>
           <t>Mixed date formats cause sorting failures, broken filters, and incorrect calculations. A date stored as text ("Jan 15, 2023") won't sort chronologically next to "2023-01-15". Downstream tools, APIs, and reports will misparse or reject inconsistent dates.</t>
         </is>
       </c>
-      <c r="I54" s="6" t="inlineStr">
+      <c r="I54" s="7" t="inlineStr">
         <is>
           <t>df["ShipDate"] = pd.to_datetime(
     df["ShipDate"], format="mixed", dayfirst=False
@@ -3230,47 +3235,47 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="inlineStr">
+      <c r="A55" s="7" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B55" s="6" t="inlineStr">
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C55" s="6" t="inlineStr">
+      <c r="C55" s="7" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D55" s="6" t="inlineStr">
+      <c r="D55" s="7" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E55" s="7" t="inlineStr">
+      <c r="E55" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F55" s="6" t="inlineStr">
+      <c r="F55" s="7" t="inlineStr">
         <is>
           <t>Inconsistent casing in categorical values</t>
         </is>
       </c>
-      <c r="G55" s="6" t="inlineStr">
+      <c r="G55" s="7" t="inlineStr">
         <is>
           <t>Shipped / shipped</t>
         </is>
       </c>
-      <c r="H55" s="6" t="inlineStr">
+      <c r="H55" s="7" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I55" s="6" t="inlineStr">
+      <c r="I55" s="7" t="inlineStr">
         <is>
           <t># Review rows where Status contains unexpected data
 mask = df["Status"].notna()
@@ -3279,47 +3284,47 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="inlineStr">
+      <c r="A56" s="7" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B56" s="6" t="inlineStr">
+      <c r="B56" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr">
+      <c r="C56" s="7" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D56" s="6" t="inlineStr">
+      <c r="D56" s="7" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E56" s="7" t="inlineStr">
+      <c r="E56" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F56" s="6" t="inlineStr">
+      <c r="F56" s="7" t="inlineStr">
         <is>
           <t>Inconsistent casing in categorical values</t>
         </is>
       </c>
-      <c r="G56" s="6" t="inlineStr">
+      <c r="G56" s="7" t="inlineStr">
         <is>
           <t>Delivered / delivered</t>
         </is>
       </c>
-      <c r="H56" s="6" t="inlineStr">
+      <c r="H56" s="7" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I56" s="6" t="inlineStr">
+      <c r="I56" s="7" t="inlineStr">
         <is>
           <t># Review rows where Status contains unexpected data
 mask = df["Status"].notna()
@@ -3328,47 +3333,47 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="inlineStr">
+      <c r="A57" s="7" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B57" s="6" t="inlineStr">
+      <c r="B57" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C57" s="6" t="inlineStr">
+      <c r="C57" s="7" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D57" s="6" t="inlineStr">
+      <c r="D57" s="7" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr">
+      <c r="E57" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F57" s="6" t="inlineStr">
+      <c r="F57" s="7" t="inlineStr">
         <is>
           <t>Inconsistent casing in categorical values</t>
         </is>
       </c>
-      <c r="G57" s="6" t="inlineStr">
+      <c r="G57" s="7" t="inlineStr">
         <is>
           <t>PENDING / Pending</t>
         </is>
       </c>
-      <c r="H57" s="6" t="inlineStr">
+      <c r="H57" s="7" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I57" s="6" t="inlineStr">
+      <c r="I57" s="7" t="inlineStr">
         <is>
           <t># Review rows where Status contains unexpected data
 mask = df["Status"].notna()
@@ -3377,47 +3382,47 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="A58" s="7" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B58" s="6" t="inlineStr">
+      <c r="B58" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr">
+      <c r="C58" s="7" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D58" s="6" t="inlineStr">
+      <c r="D58" s="7" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E58" s="9" t="inlineStr">
+      <c r="E58" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F58" s="6" t="inlineStr">
+      <c r="F58" s="7" t="inlineStr">
         <is>
           <t>Placeholder "Test" found 2 times</t>
         </is>
       </c>
-      <c r="G58" s="6" t="inlineStr">
+      <c r="G58" s="7" t="inlineStr">
         <is>
           <t>20.0% of non-null values</t>
         </is>
       </c>
-      <c r="H58" s="6" t="inlineStr">
+      <c r="H58" s="7" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I58" s="6" t="inlineStr">
+      <c r="I58" s="7" t="inlineStr">
         <is>
           <t>import numpy as np
 df["Status"] = df["Status"].replace("Test", np.nan)</t>
@@ -3425,94 +3430,94 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="inlineStr">
+      <c r="A59" s="7" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B59" s="6" t="inlineStr">
+      <c r="B59" s="7" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C59" s="6" t="inlineStr">
+      <c r="C59" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D59" s="6" t="inlineStr">
+      <c r="D59" s="7" t="inlineStr">
         <is>
           <t>Exact Duplicate</t>
         </is>
       </c>
-      <c r="E59" s="7" t="inlineStr">
+      <c r="E59" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F59" s="6" t="inlineStr">
+      <c r="F59" s="7" t="inlineStr">
         <is>
           <t>2 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G59" s="6" t="inlineStr">
+      <c r="G59" s="7" t="inlineStr">
         <is>
           <t>Rows: 5, 6</t>
         </is>
       </c>
-      <c r="H59" s="6" t="inlineStr">
+      <c r="H59" s="7" t="inlineStr">
         <is>
           <t>Exact duplicate rows are the clearest sign of a data quality issue — they can result from double-submissions, ETL failures, or missing unique constraints. Every duplicate inflates counts and distorts any metric built on this data.</t>
         </is>
       </c>
-      <c r="I59" s="6" t="inlineStr">
+      <c r="I59" s="7" t="inlineStr">
         <is>
           <t>df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="inlineStr">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B60" s="7" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C60" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D60" s="6" t="inlineStr">
+      <c r="D60" s="7" t="inlineStr">
         <is>
           <t>Exact Duplicate</t>
         </is>
       </c>
-      <c r="E60" s="7" t="inlineStr">
+      <c r="E60" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F60" s="6" t="inlineStr">
+      <c r="F60" s="7" t="inlineStr">
         <is>
           <t>2 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G60" s="6" t="inlineStr">
+      <c r="G60" s="7" t="inlineStr">
         <is>
           <t>Rows: 7, 8</t>
         </is>
       </c>
-      <c r="H60" s="6" t="inlineStr">
+      <c r="H60" s="7" t="inlineStr">
         <is>
           <t>Exact duplicate rows are the clearest sign of a data quality issue — they can result from double-submissions, ETL failures, or missing unique constraints. Every duplicate inflates counts and distorts any metric built on this data.</t>
         </is>
       </c>
-      <c r="I60" s="6" t="inlineStr">
+      <c r="I60" s="7" t="inlineStr">
         <is>
           <t>df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
         </is>

</xml_diff>

<commit_message>
Extract shared palette module, add brand tests, and type annotations
Centralizes all Lailara color tokens in palette.py so HTML, PDF, and
Excel generators reference one source of truth instead of duplicating
hex values. Adds 12 branding tests that verify palette colors appear
in output and no legacy colors remain. Adds type annotations to all
public reporting functions. Fixes design system path in CLAUDE.md.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/output/sample_messy_data_audit_findings.xlsx
+++ b/samples/output/sample_messy_data_audit_findings.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,10 +51,6 @@
     <font>
       <name val="Source Sans Pro"/>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -112,12 +108,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -545,7 +540,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-20 11:12:08</t>
+          <t>2026-05-20 11:28:11</t>
         </is>
       </c>
     </row>
@@ -565,7 +560,7 @@
           <t>Sheet: Customers</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Score: 0/100</t>
         </is>
@@ -577,7 +572,7 @@
           <t>Sheet: Orders</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Score: 65/100</t>
         </is>
@@ -609,94 +604,94 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Inferred Type</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Issue Type</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Example / Detail</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Why It Matters</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>Suggested Fix</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>CustomerID</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Mixed ID formats</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>29 coded (e.g. CUST-001) vs 1 bare numbers</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>df["_CustomerID_format"] = df["CustomerID"].apply(
     lambda x: "coded" if isinstance(x, str)
@@ -706,94 +701,94 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>FirstName</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>df["FirstName"] = df["FirstName"].fillna(df["FirstName"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>FirstName</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Code/ID stuffed in name field</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>REF-4421</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t># Review rows where FirstName contains unexpected data
 mask = df["FirstName"].notna()
@@ -802,47 +797,47 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>FirstName</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Placeholder "Test" found 3 times</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>import numpy as np
 df["FirstName"] = df["FirstName"].replace("Test", np.nan)</t>
@@ -850,47 +845,47 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>FirstName</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>import numpy as np
 df["FirstName"] = df["FirstName"].replace("TBD", np.nan)</t>
@@ -898,94 +893,94 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>LastName</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>df["LastName"] = df["LastName"].fillna(df["LastName"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>LastName</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>import numpy as np
 df["LastName"] = df["LastName"].replace("TBD", np.nan)</t>
@@ -993,47 +988,47 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>LastName</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>"User" repeated 3 times</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>df["_LastName_review"] = (
     df["LastName"] == "User"
@@ -1042,47 +1037,47 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>LastName</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>"Doe" repeated 3 times</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>df["_LastName_review"] = (
     df["LastName"] == "Doe"
@@ -1091,94 +1086,94 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>df["Email"] = df["Email"].fillna(df["Email"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Invalid email format</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>henrylee</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>email_re = r"^[a-zA-Z0-9._%+-]+@[a-zA-Z0-9.-]+\.[a-zA-Z]{2,}$"
 df["_Email_invalid"] = ~df["Email"].str.match(
@@ -1188,47 +1183,47 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Invalid email format</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>nancy w@example.com</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>email_re = r"^[a-zA-Z0-9._%+-]+@[a-zA-Z0-9.-]+\.[a-zA-Z]{2,}$"
 df["_Email_invalid"] = ~df["Email"].str.match(
@@ -1238,47 +1233,47 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>"test@test.com" repeated 3 times</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>df["_Email_review"] = (
     df["Email"] == "test@test.com"
@@ -1287,94 +1282,94 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>df["Phone"] = df["Phone"].fillna(df["Phone"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Mixed phone formats: 17 values deviate from (XXX) XXX-XXXX</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>(XXX) XXX-XXXX: 9; XXX-XXX-XXXX: 8; (non-standard): 3; +1-XXX-XXX-XXXX: 2; XXXXXXXXXX: 1; XXX.XXX.XXXX: 1; XXX XXX XXXX: 1; (XXX)XXXXXXX: 1</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Inconsistent phone formats break deduplication, prevent reliable search/lookup, and cause issues with automated dialers or SMS systems. Two records for the same person may appear as different contacts if one says "(555) 123-4567" and another says "5551234567".</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>digits = df["Phone"].str.replace(r"\D", "", regex=True)
 digits = digits.str.slice(-10)
@@ -1386,47 +1381,47 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>import numpy as np
 df["Phone"] = df["Phone"].replace("TBD", np.nan)</t>
@@ -1434,47 +1429,47 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>"(555) 123-4567" repeated 3 times</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I18" s="7" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>df["_Phone_review"] = (
     df["Phone"] == "(555) 123-4567"
@@ -1483,47 +1478,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>"000-000-0000" repeated 3 times</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I19" s="7" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>df["_Phone_review"] = (
     df["Phone"] == "000-000-0000"
@@ -1532,47 +1527,47 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>"555-555-5555" repeated 3 times</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I20" s="7" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>df["_Phone_review"] = (
     df["Phone"] == "555-555-5555"
@@ -1581,94 +1576,94 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>df["JoinDate"] = df["JoinDate"].fillna(df["JoinDate"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>Mixed date formats: 12 values deviate from YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>YYYY-MM-DD: 14; MM/DD/YYYY: 3; Mon DD, YYYY: 3; (non-standard): 1; YYYY/MM/DD: 1; M/D/YYYY: 1; DD-Mon-YYYY: 1; YYYY.MM.DD: 1; MM-DD-YYYY: 1</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>Mixed date formats cause sorting failures, broken filters, and incorrect calculations. A date stored as text ("Jan 15, 2023") won't sort chronologically next to "2023-01-15". Downstream tools, APIs, and reports will misparse or reject inconsistent dates.</t>
         </is>
       </c>
-      <c r="I22" s="7" t="inlineStr">
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>df["JoinDate"] = pd.to_datetime(
     df["JoinDate"], format="mixed", dayfirst=False
@@ -1677,47 +1672,47 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I23" s="7" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>import numpy as np
 df["JoinDate"] = df["JoinDate"].replace("TBD", np.nan)</t>
@@ -1725,47 +1720,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>"2023-01-01" repeated 6 times</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>23.1% of non-null values</t>
         </is>
       </c>
-      <c r="H24" s="7" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I24" s="7" t="inlineStr">
+      <c r="I24" s="6" t="inlineStr">
         <is>
           <t>df["_JoinDate_review"] = (
     df["JoinDate"] == "2023-01-01"
@@ -1774,47 +1769,47 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>JoinDate</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>"2023-01-15" repeated 3 times</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I25" s="7" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>df["_JoinDate_review"] = (
     df["JoinDate"] == "2023-01-15"
@@ -1823,94 +1818,94 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H26" s="7" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I26" s="7" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>df["AccountBalance"] = df["AccountBalance"].fillna(df["AccountBalance"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>Mixed currency formats: 11 values deviate from $X,XXX.XX</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>$X,XXX.XX: 15; X,XXX.XX (no symbol): 4; $X,XXX: 3; (non-standard): 2; $X,XXX.XX USD: 2</t>
         </is>
       </c>
-      <c r="H27" s="7" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>Mixed currency formats ("$1,250.00" vs "1250" vs "five thousand") prevent accurate aggregation and comparison. Summing a column with text-formatted currency returns errors or silently drops values, leading to wrong totals in financial reports.</t>
         </is>
       </c>
-      <c r="I27" s="7" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>df["AccountBalance"] = (
     df["AccountBalance"].str.replace(r"[^\d.]", "", regex=True)
@@ -1920,47 +1915,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E28" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>Text in currency field</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I28" s="7" t="inlineStr">
+      <c r="I28" s="6" t="inlineStr">
         <is>
           <t>df["_AccountBalance_invalid"] = ~df["AccountBalance"].str.match(
     r"^[\$\d,\.\-]+$", na=False
@@ -1969,47 +1964,47 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E29" s="8" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>Text in currency field</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>five thousand</t>
         </is>
       </c>
-      <c r="H29" s="7" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I29" s="7" t="inlineStr">
+      <c r="I29" s="6" t="inlineStr">
         <is>
           <t>df["_AccountBalance_invalid"] = ~df["AccountBalance"].str.match(
     r"^[\$\d,\.\-]+$", na=False
@@ -2018,47 +2013,47 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="E30" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G30" s="6" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I30" s="7" t="inlineStr">
+      <c r="I30" s="6" t="inlineStr">
         <is>
           <t>import numpy as np
 df["AccountBalance"] = df["AccountBalance"].replace("TBD", np.nan)</t>
@@ -2066,47 +2061,47 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E31" s="8" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>"$0.00" repeated 6 times</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>23.1% of non-null values</t>
         </is>
       </c>
-      <c r="H31" s="7" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I31" s="7" t="inlineStr">
+      <c r="I31" s="6" t="inlineStr">
         <is>
           <t>df["_AccountBalance_review"] = (
     df["AccountBalance"] == "$0.00"
@@ -2115,47 +2110,47 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>AccountBalance</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E32" s="10" t="inlineStr">
+      <c r="E32" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>"$1,250.00" repeated 3 times</t>
         </is>
       </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H32" s="7" t="inlineStr">
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I32" s="7" t="inlineStr">
+      <c r="I32" s="6" t="inlineStr">
         <is>
           <t>df["_AccountBalance_review"] = (
     df["AccountBalance"] == "$1,250.00"
@@ -2164,94 +2159,94 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E33" s="9" t="inlineStr">
+      <c r="E33" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G33" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H33" s="7" t="inlineStr">
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I33" s="7" t="inlineStr">
+      <c r="I33" s="6" t="inlineStr">
         <is>
           <t>df["Status"] = df["Status"].fillna(df["Status"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
+      <c r="E34" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>Inconsistent casing in categorical values</t>
         </is>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="G34" s="6" t="inlineStr">
         <is>
           <t>ACTIVE / Active / active</t>
         </is>
       </c>
-      <c r="H34" s="7" t="inlineStr">
+      <c r="H34" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I34" s="7" t="inlineStr">
+      <c r="I34" s="6" t="inlineStr">
         <is>
           <t># Review rows where Status contains unexpected data
 mask = df["Status"].notna()
@@ -2260,47 +2255,47 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F35" s="7" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G35" s="7" t="inlineStr">
+      <c r="G35" s="6" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H35" s="7" t="inlineStr">
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I35" s="7" t="inlineStr">
+      <c r="I35" s="6" t="inlineStr">
         <is>
           <t>import numpy as np
 df["Status"] = df["Status"].replace("TBD", np.nan)</t>
@@ -2308,47 +2303,47 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E36" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <t>"Active" repeated 18 times</t>
         </is>
       </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="G36" s="6" t="inlineStr">
         <is>
           <t>69.2% of non-null values</t>
         </is>
       </c>
-      <c r="H36" s="7" t="inlineStr">
+      <c r="H36" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I36" s="7" t="inlineStr">
+      <c r="I36" s="6" t="inlineStr">
         <is>
           <t>df["_Status_review"] = (
     df["Status"] == "Active"
@@ -2357,94 +2352,94 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="E37" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F37" s="7" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>4 of 30 values missing (13.3%)</t>
         </is>
       </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="G37" s="6" t="inlineStr">
         <is>
           <t>Null: 3, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H37" s="7" t="inlineStr">
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I37" s="7" t="inlineStr">
+      <c r="I37" s="6" t="inlineStr">
         <is>
           <t>df["ZipCode"] = df["ZipCode"].fillna(df["ZipCode"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B38" s="7" t="inlineStr">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D38" s="7" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E38" s="10" t="inlineStr">
+      <c r="E38" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>Placeholder "00000" found 3 times</t>
         </is>
       </c>
-      <c r="G38" s="7" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H38" s="7" t="inlineStr">
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I38" s="7" t="inlineStr">
+      <c r="I38" s="6" t="inlineStr">
         <is>
           <t>import numpy as np
 df["ZipCode"] = df["ZipCode"].replace("00000", np.nan)</t>
@@ -2452,47 +2447,47 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="inlineStr">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E39" s="9" t="inlineStr">
+      <c r="E39" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G39" s="7" t="inlineStr">
+      <c r="G39" s="6" t="inlineStr">
         <is>
           <t>3.8% of non-null values</t>
         </is>
       </c>
-      <c r="H39" s="7" t="inlineStr">
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I39" s="7" t="inlineStr">
+      <c r="I39" s="6" t="inlineStr">
         <is>
           <t>import numpy as np
 df["ZipCode"] = df["ZipCode"].replace("TBD", np.nan)</t>
@@ -2500,47 +2495,47 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B40" s="7" t="inlineStr">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E40" s="10" t="inlineStr">
+      <c r="E40" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F40" s="7" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>"30301" repeated 3 times</t>
         </is>
       </c>
-      <c r="G40" s="7" t="inlineStr">
+      <c r="G40" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H40" s="7" t="inlineStr">
+      <c r="H40" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I40" s="7" t="inlineStr">
+      <c r="I40" s="6" t="inlineStr">
         <is>
           <t>df["_ZipCode_review"] = (
     df["ZipCode"] == "30301"
@@ -2549,47 +2544,47 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>ZipCode</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E41" s="10" t="inlineStr">
+      <c r="E41" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>"12345" repeated 3 times</t>
         </is>
       </c>
-      <c r="G41" s="7" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>11.5% of non-null values</t>
         </is>
       </c>
-      <c r="H41" s="7" t="inlineStr">
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I41" s="7" t="inlineStr">
+      <c r="I41" s="6" t="inlineStr">
         <is>
           <t>df["_ZipCode_review"] = (
     df["ZipCode"] == "12345"
@@ -2598,47 +2593,47 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B42" s="7" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>freetext</t>
         </is>
       </c>
-      <c r="D42" s="7" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E42" s="10" t="inlineStr">
+      <c r="E42" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>15 of 30 values missing (50.0%)</t>
         </is>
       </c>
-      <c r="G42" s="7" t="inlineStr">
+      <c r="G42" s="6" t="inlineStr">
         <is>
           <t>Null: 14, Blank: 0, Whitespace: 1</t>
         </is>
       </c>
-      <c r="H42" s="7" t="inlineStr">
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I42" s="7" t="inlineStr">
+      <c r="I42" s="6" t="inlineStr">
         <is>
           <t># Option A: Fill with most common value
 df["Notes"] = df["Notes"].fillna(df["Notes"].mode()[0])
@@ -2648,47 +2643,47 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B43" s="7" t="inlineStr">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>freetext</t>
         </is>
       </c>
-      <c r="D43" s="7" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E43" s="10" t="inlineStr">
+      <c r="E43" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F43" s="7" t="inlineStr">
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TEST" found 3 times</t>
         </is>
       </c>
-      <c r="G43" s="7" t="inlineStr">
+      <c r="G43" s="6" t="inlineStr">
         <is>
           <t>20.0% of non-null values</t>
         </is>
       </c>
-      <c r="H43" s="7" t="inlineStr">
+      <c r="H43" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I43" s="7" t="inlineStr">
+      <c r="I43" s="6" t="inlineStr">
         <is>
           <t>import numpy as np
 df["Notes"] = df["Notes"].replace("TEST", np.nan)</t>
@@ -2696,47 +2691,47 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B44" s="7" t="inlineStr">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr">
+      <c r="C44" s="6" t="inlineStr">
         <is>
           <t>freetext</t>
         </is>
       </c>
-      <c r="D44" s="7" t="inlineStr">
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E44" s="10" t="inlineStr">
+      <c r="E44" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F44" s="7" t="inlineStr">
+      <c r="F44" s="6" t="inlineStr">
         <is>
           <t>Placeholder "TBD" found 1 times</t>
         </is>
       </c>
-      <c r="G44" s="7" t="inlineStr">
+      <c r="G44" s="6" t="inlineStr">
         <is>
           <t>6.7% of non-null values</t>
         </is>
       </c>
-      <c r="H44" s="7" t="inlineStr">
+      <c r="H44" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I44" s="7" t="inlineStr">
+      <c r="I44" s="6" t="inlineStr">
         <is>
           <t>import numpy as np
 df["Notes"] = df["Notes"].replace("TBD", np.nan)</t>
@@ -2744,47 +2739,47 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>freetext</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>suspicious_repetition</t>
         </is>
       </c>
-      <c r="E45" s="10" t="inlineStr">
+      <c r="E45" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>"Preferred customer" repeated 3 times</t>
         </is>
       </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="G45" s="6" t="inlineStr">
         <is>
           <t>20.0% of non-null values</t>
         </is>
       </c>
-      <c r="H45" s="7" t="inlineStr">
+      <c r="H45" s="6" t="inlineStr">
         <is>
           <t>When the same value appears far more often than expected, it may indicate a default value that was never updated, a copy-paste error, or a system glitch that stamped the same data across multiple records.</t>
         </is>
       </c>
-      <c r="I45" s="7" t="inlineStr">
+      <c r="I45" s="6" t="inlineStr">
         <is>
           <t>df["_Notes_review"] = (
     df["Notes"] == "Preferred customer"
@@ -2793,47 +2788,47 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B46" s="7" t="inlineStr">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C46" s="7" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D46" s="7" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>Phantom Duplicate</t>
         </is>
       </c>
-      <c r="E46" s="10" t="inlineStr">
+      <c r="E46" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <t>3 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G46" s="7" t="inlineStr">
+      <c r="G46" s="6" t="inlineStr">
         <is>
           <t>Rows: 2, 8, 9</t>
         </is>
       </c>
-      <c r="H46" s="7" t="inlineStr">
+      <c r="H46" s="6" t="inlineStr">
         <is>
           <t>These records look different on the surface (different casing, extra spaces, punctuation variations) but represent the same entity. They cause inflated counts, split transaction histories, and duplicate outreach — problems that compound over time.</t>
         </is>
       </c>
-      <c r="I46" s="7" t="inlineStr">
+      <c r="I46" s="6" t="inlineStr">
         <is>
           <t># Normalize text columns before deduplication
 text_cols = df.select_dtypes(include="object").columns
@@ -2844,47 +2839,47 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D47" s="7" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Phantom Duplicate</t>
         </is>
       </c>
-      <c r="E47" s="10" t="inlineStr">
+      <c r="E47" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <t>2 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G47" s="7" t="inlineStr">
+      <c r="G47" s="6" t="inlineStr">
         <is>
           <t>Rows: 3, 10</t>
         </is>
       </c>
-      <c r="H47" s="7" t="inlineStr">
+      <c r="H47" s="6" t="inlineStr">
         <is>
           <t>These records look different on the surface (different casing, extra spaces, punctuation variations) but represent the same entity. They cause inflated counts, split transaction histories, and duplicate outreach — problems that compound over time.</t>
         </is>
       </c>
-      <c r="I47" s="7" t="inlineStr">
+      <c r="I47" s="6" t="inlineStr">
         <is>
           <t># Normalize text columns before deduplication
 text_cols = df.select_dtypes(include="object").columns
@@ -2895,94 +2890,94 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D48" s="7" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>Exact Duplicate</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr">
+      <c r="E48" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr">
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>3 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="G48" s="6" t="inlineStr">
         <is>
           <t>Rows: 11, 12, 13</t>
         </is>
       </c>
-      <c r="H48" s="7" t="inlineStr">
+      <c r="H48" s="6" t="inlineStr">
         <is>
           <t>Exact duplicate rows are the clearest sign of a data quality issue — they can result from double-submissions, ETL failures, or missing unique constraints. Every duplicate inflates counts and distorts any metric built on this data.</t>
         </is>
       </c>
-      <c r="I48" s="7" t="inlineStr">
+      <c r="I48" s="6" t="inlineStr">
         <is>
           <t>df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B49" s="7" t="inlineStr">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C49" s="7" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D49" s="7" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>Phantom Duplicate</t>
         </is>
       </c>
-      <c r="E49" s="8" t="inlineStr">
+      <c r="E49" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F49" s="7" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>4 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G49" s="7" t="inlineStr">
+      <c r="G49" s="6" t="inlineStr">
         <is>
           <t>Rows: 14, 19, 20, 21</t>
         </is>
       </c>
-      <c r="H49" s="7" t="inlineStr">
+      <c r="H49" s="6" t="inlineStr">
         <is>
           <t>These records look different on the surface (different casing, extra spaces, punctuation variations) but represent the same entity. They cause inflated counts, split transaction histories, and duplicate outreach — problems that compound over time.</t>
         </is>
       </c>
-      <c r="I49" s="7" t="inlineStr">
+      <c r="I49" s="6" t="inlineStr">
         <is>
           <t># Normalize text columns before deduplication
 text_cols = df.select_dtypes(include="object").columns
@@ -2993,94 +2988,94 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D50" s="7" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>Exact Duplicate</t>
         </is>
       </c>
-      <c r="E50" s="8" t="inlineStr">
+      <c r="E50" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F50" s="7" t="inlineStr">
+      <c r="F50" s="6" t="inlineStr">
         <is>
           <t>2 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="G50" s="6" t="inlineStr">
         <is>
           <t>Rows: 25, 27</t>
         </is>
       </c>
-      <c r="H50" s="7" t="inlineStr">
+      <c r="H50" s="6" t="inlineStr">
         <is>
           <t>Exact duplicate rows are the clearest sign of a data quality issue — they can result from double-submissions, ETL failures, or missing unique constraints. Every duplicate inflates counts and distorts any metric built on this data.</t>
         </is>
       </c>
-      <c r="I50" s="7" t="inlineStr">
+      <c r="I50" s="6" t="inlineStr">
         <is>
           <t>df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="inlineStr">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B51" s="7" t="inlineStr">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>OrderDate</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E51" s="8" t="inlineStr">
+      <c r="E51" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
+      <c r="F51" s="6" t="inlineStr">
         <is>
           <t>Mixed date formats: 4 values deviate from YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="G51" s="7" t="inlineStr">
+      <c r="G51" s="6" t="inlineStr">
         <is>
           <t>YYYY-MM-DD: 6; MM/DD/YYYY: 1; Mon DD, YYYY: 1; M/D/YYYY: 1; YYYY/MM/DD: 1</t>
         </is>
       </c>
-      <c r="H51" s="7" t="inlineStr">
+      <c r="H51" s="6" t="inlineStr">
         <is>
           <t>Mixed date formats cause sorting failures, broken filters, and incorrect calculations. A date stored as text ("Jan 15, 2023") won't sort chronologically next to "2023-01-15". Downstream tools, APIs, and reports will misparse or reject inconsistent dates.</t>
         </is>
       </c>
-      <c r="I51" s="7" t="inlineStr">
+      <c r="I51" s="6" t="inlineStr">
         <is>
           <t>df["OrderDate"] = pd.to_datetime(
     df["OrderDate"], format="mixed", dayfirst=False
@@ -3089,47 +3084,47 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="inlineStr">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B52" s="7" t="inlineStr">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="C52" s="7" t="inlineStr">
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D52" s="7" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E52" s="10" t="inlineStr">
+      <c r="E52" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <t>Mixed currency formats: 3 values deviate from $X,XXX.XX</t>
         </is>
       </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>$X,XXX.XX: 7; X,XXX (bare number): 2; $X,XXX: 1</t>
         </is>
       </c>
-      <c r="H52" s="7" t="inlineStr">
+      <c r="H52" s="6" t="inlineStr">
         <is>
           <t>Mixed currency formats ("$1,250.00" vs "1250" vs "five thousand") prevent accurate aggregation and comparison. Summing a column with text-formatted currency returns errors or silently drops values, leading to wrong totals in financial reports.</t>
         </is>
       </c>
-      <c r="I52" s="7" t="inlineStr">
+      <c r="I52" s="6" t="inlineStr">
         <is>
           <t>df["Amount"] = (
     df["Amount"].str.replace(r"[^\d.]", "", regex=True)
@@ -3139,94 +3134,94 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B53" s="7" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>ShipDate</t>
         </is>
       </c>
-      <c r="C53" s="7" t="inlineStr">
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D53" s="7" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>null_analysis</t>
         </is>
       </c>
-      <c r="E53" s="9" t="inlineStr">
+      <c r="E53" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F53" s="7" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>2 of 10 values missing (20.0%)</t>
         </is>
       </c>
-      <c r="G53" s="7" t="inlineStr">
+      <c r="G53" s="6" t="inlineStr">
         <is>
           <t>Null: 2, Blank: 0, Whitespace: 0</t>
         </is>
       </c>
-      <c r="H53" s="7" t="inlineStr">
+      <c r="H53" s="6" t="inlineStr">
         <is>
           <t>High rates of missing data reduce the reliability of any analysis built on this field. Missing values can skew averages, break joins between tables, and cause downstream systems to error out or produce incomplete results.</t>
         </is>
       </c>
-      <c r="I53" s="7" t="inlineStr">
+      <c r="I53" s="6" t="inlineStr">
         <is>
           <t>df["ShipDate"] = df["ShipDate"].fillna(df["ShipDate"].mode()[0])</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="7" t="inlineStr">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B54" s="7" t="inlineStr">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>ShipDate</t>
         </is>
       </c>
-      <c r="C54" s="7" t="inlineStr">
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D54" s="7" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>mixed_format</t>
         </is>
       </c>
-      <c r="E54" s="8" t="inlineStr">
+      <c r="E54" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F54" s="7" t="inlineStr">
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <t>Mixed date formats: 3 values deviate from YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="G54" s="7" t="inlineStr">
+      <c r="G54" s="6" t="inlineStr">
         <is>
           <t>YYYY-MM-DD: 5; MM/DD/YYYY: 1; Mon DD, YYYY: 1; M/D/YYYY: 1</t>
         </is>
       </c>
-      <c r="H54" s="7" t="inlineStr">
+      <c r="H54" s="6" t="inlineStr">
         <is>
           <t>Mixed date formats cause sorting failures, broken filters, and incorrect calculations. A date stored as text ("Jan 15, 2023") won't sort chronologically next to "2023-01-15". Downstream tools, APIs, and reports will misparse or reject inconsistent dates.</t>
         </is>
       </c>
-      <c r="I54" s="7" t="inlineStr">
+      <c r="I54" s="6" t="inlineStr">
         <is>
           <t>df["ShipDate"] = pd.to_datetime(
     df["ShipDate"], format="mixed", dayfirst=False
@@ -3235,47 +3230,47 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="inlineStr">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C55" s="7" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D55" s="7" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E55" s="8" t="inlineStr">
+      <c r="E55" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>Inconsistent casing in categorical values</t>
         </is>
       </c>
-      <c r="G55" s="7" t="inlineStr">
+      <c r="G55" s="6" t="inlineStr">
         <is>
           <t>Shipped / shipped</t>
         </is>
       </c>
-      <c r="H55" s="7" t="inlineStr">
+      <c r="H55" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I55" s="7" t="inlineStr">
+      <c r="I55" s="6" t="inlineStr">
         <is>
           <t># Review rows where Status contains unexpected data
 mask = df["Status"].notna()
@@ -3284,47 +3279,47 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="inlineStr">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B56" s="7" t="inlineStr">
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C56" s="7" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D56" s="7" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E56" s="8" t="inlineStr">
+      <c r="E56" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
+      <c r="F56" s="6" t="inlineStr">
         <is>
           <t>Inconsistent casing in categorical values</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G56" s="6" t="inlineStr">
         <is>
           <t>Delivered / delivered</t>
         </is>
       </c>
-      <c r="H56" s="7" t="inlineStr">
+      <c r="H56" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I56" s="7" t="inlineStr">
+      <c r="I56" s="6" t="inlineStr">
         <is>
           <t># Review rows where Status contains unexpected data
 mask = df["Status"].notna()
@@ -3333,47 +3328,47 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="inlineStr">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B57" s="7" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C57" s="7" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>wrong_purpose</t>
         </is>
       </c>
-      <c r="E57" s="8" t="inlineStr">
+      <c r="E57" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F57" s="7" t="inlineStr">
+      <c r="F57" s="6" t="inlineStr">
         <is>
           <t>Inconsistent casing in categorical values</t>
         </is>
       </c>
-      <c r="G57" s="7" t="inlineStr">
+      <c r="G57" s="6" t="inlineStr">
         <is>
           <t>PENDING / Pending</t>
         </is>
       </c>
-      <c r="H57" s="7" t="inlineStr">
+      <c r="H57" s="6" t="inlineStr">
         <is>
           <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
         </is>
       </c>
-      <c r="I57" s="7" t="inlineStr">
+      <c r="I57" s="6" t="inlineStr">
         <is>
           <t># Review rows where Status contains unexpected data
 mask = df["Status"].notna()
@@ -3382,47 +3377,47 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="inlineStr">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B58" s="7" t="inlineStr">
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C58" s="7" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D58" s="7" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>placeholder_value</t>
         </is>
       </c>
-      <c r="E58" s="10" t="inlineStr">
+      <c r="E58" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F58" s="7" t="inlineStr">
+      <c r="F58" s="6" t="inlineStr">
         <is>
           <t>Placeholder "Test" found 2 times</t>
         </is>
       </c>
-      <c r="G58" s="7" t="inlineStr">
+      <c r="G58" s="6" t="inlineStr">
         <is>
           <t>20.0% of non-null values</t>
         </is>
       </c>
-      <c r="H58" s="7" t="inlineStr">
+      <c r="H58" s="6" t="inlineStr">
         <is>
           <t>Placeholder values ("Test", "N/A", "TBD") that persist in production data inflate counts, skew averages, and create phantom records. They often indicate incomplete data entry or inadequate validation at the point of capture.</t>
         </is>
       </c>
-      <c r="I58" s="7" t="inlineStr">
+      <c r="I58" s="6" t="inlineStr">
         <is>
           <t>import numpy as np
 df["Status"] = df["Status"].replace("Test", np.nan)</t>
@@ -3430,94 +3425,94 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="inlineStr">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B59" s="7" t="inlineStr">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C59" s="7" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D59" s="7" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>Exact Duplicate</t>
         </is>
       </c>
-      <c r="E59" s="8" t="inlineStr">
+      <c r="E59" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F59" s="7" t="inlineStr">
+      <c r="F59" s="6" t="inlineStr">
         <is>
           <t>2 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G59" s="7" t="inlineStr">
+      <c r="G59" s="6" t="inlineStr">
         <is>
           <t>Rows: 5, 6</t>
         </is>
       </c>
-      <c r="H59" s="7" t="inlineStr">
+      <c r="H59" s="6" t="inlineStr">
         <is>
           <t>Exact duplicate rows are the clearest sign of a data quality issue — they can result from double-submissions, ETL failures, or missing unique constraints. Every duplicate inflates counts and distorts any metric built on this data.</t>
         </is>
       </c>
-      <c r="I59" s="7" t="inlineStr">
+      <c r="I59" s="6" t="inlineStr">
         <is>
           <t>df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="7" t="inlineStr">
+      <c r="A60" s="6" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="B60" s="7" t="inlineStr">
+      <c r="B60" s="6" t="inlineStr">
         <is>
           <t>(row-level)</t>
         </is>
       </c>
-      <c r="C60" s="7" t="inlineStr">
+      <c r="C60" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D60" s="7" t="inlineStr">
+      <c r="D60" s="6" t="inlineStr">
         <is>
           <t>Exact Duplicate</t>
         </is>
       </c>
-      <c r="E60" s="8" t="inlineStr">
+      <c r="E60" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F60" s="7" t="inlineStr">
+      <c r="F60" s="6" t="inlineStr">
         <is>
           <t>2 rows appear to be the same record</t>
         </is>
       </c>
-      <c r="G60" s="7" t="inlineStr">
+      <c r="G60" s="6" t="inlineStr">
         <is>
           <t>Rows: 7, 8</t>
         </is>
       </c>
-      <c r="H60" s="7" t="inlineStr">
+      <c r="H60" s="6" t="inlineStr">
         <is>
           <t>Exact duplicate rows are the clearest sign of a data quality issue — they can result from double-submissions, ETL failures, or missing unique constraints. Every duplicate inflates counts and distorts any metric built on this data.</t>
         </is>
       </c>
-      <c r="I60" s="7" t="inlineStr">
+      <c r="I60" s="6" t="inlineStr">
         <is>
           <t>df = df.drop_duplicates(keep="first").reset_index(drop=True)</t>
         </is>

</xml_diff>

<commit_message>
fix(profile,findings): guard numeric range + ID-format why-text; regenerate samples; move dev docs
- _compute_profile no longer emits min/max/mean/median for id/currency
  columns unless >=80% of non-empty values parse as numeric, killing the
  meaningless 'range 1027.0-1027.0' output when a lone number sits among
  coded IDs (e.g. CUST-001).
- The 'Mixed ID formats' finding now routes to a dedicated why-matters
  entry about broken joins/lookups/dedup instead of the generic
  wrong-purpose (field-misuse) text.
- Regenerate committed sample report/findings to reflect both fixes.
- Move dev-only docs (CLAUDE/HANDOFF/PLAN/DECISIONS/AUDIT) into .dev/ so
  the public root shows only README, CHANGELOG, RELEASING, LICENSE, source,
  samples, tests.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/output/sample_messy_data_audit_findings.xlsx
+++ b/samples/output/sample_messy_data_audit_findings.xlsx
@@ -540,7 +540,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-20 11:28:11</t>
+          <t>2026-07-07 18:48:43</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -649,6 +649,16 @@
           <t>Suggested Fix</t>
         </is>
       </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Cardinality</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Uniqueness %</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -688,7 +698,7 @@
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>When a field is used for something other than its intended purpose — like storing reference codes in a name field or text in a currency field — it corrupts both the misused field and whatever field should have held that data. This makes the data unreliable for any analysis.</t>
+          <t>Inconsistent ID formats break joins, lookups, and deduplication — a key stored as "CUST-001" won't match "1027", so related records silently fail to link.</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr">
@@ -699,6 +709,12 @@
 )</t>
         </is>
       </c>
+      <c r="J2" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="K2" s="6" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -745,6 +761,12 @@
         <is>
           <t>df["FirstName"] = df["FirstName"].fillna(df["FirstName"].mode()[0])</t>
         </is>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>80.8</v>
       </c>
     </row>
     <row r="4">
@@ -795,6 +817,12 @@
 suspect = df.loc[mask, "FirstName"]</t>
         </is>
       </c>
+      <c r="J4" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>80.8</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -843,6 +871,12 @@
 df["FirstName"] = df["FirstName"].replace("Test", np.nan)</t>
         </is>
       </c>
+      <c r="J5" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>80.8</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -891,6 +925,12 @@
 df["FirstName"] = df["FirstName"].replace("TBD", np.nan)</t>
         </is>
       </c>
+      <c r="J6" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>80.8</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -938,6 +978,12 @@
           <t>df["LastName"] = df["LastName"].fillna(df["LastName"].mode()[0])</t>
         </is>
       </c>
+      <c r="J7" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>76.90000000000001</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -985,6 +1031,12 @@
           <t>import numpy as np
 df["LastName"] = df["LastName"].replace("TBD", np.nan)</t>
         </is>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -1035,6 +1087,12 @@
 )</t>
         </is>
       </c>
+      <c r="J9" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>76.90000000000001</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -1084,6 +1142,12 @@
 )</t>
         </is>
       </c>
+      <c r="J10" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>76.90000000000001</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -1130,6 +1194,12 @@
         <is>
           <t>df["Email"] = df["Email"].fillna(df["Email"].mode()[0])</t>
         </is>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>80.8</v>
       </c>
     </row>
     <row r="12">
@@ -1181,6 +1251,12 @@
 )</t>
         </is>
       </c>
+      <c r="J12" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>80.8</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -1231,6 +1307,12 @@
 )</t>
         </is>
       </c>
+      <c r="J13" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>80.8</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -1280,6 +1362,12 @@
 )</t>
         </is>
       </c>
+      <c r="J14" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>80.8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -1326,6 +1414,12 @@
         <is>
           <t>df["Phone"] = df["Phone"].fillna(df["Phone"].mode()[0])</t>
         </is>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>73.09999999999999</v>
       </c>
     </row>
     <row r="16">
@@ -1379,6 +1473,12 @@
 )</t>
         </is>
       </c>
+      <c r="J16" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>73.09999999999999</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -1426,6 +1526,12 @@
           <t>import numpy as np
 df["Phone"] = df["Phone"].replace("TBD", np.nan)</t>
         </is>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>73.09999999999999</v>
       </c>
     </row>
     <row r="18">
@@ -1476,6 +1582,12 @@
 )</t>
         </is>
       </c>
+      <c r="J18" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>73.09999999999999</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -1525,6 +1637,12 @@
 )</t>
         </is>
       </c>
+      <c r="J19" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>73.09999999999999</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1574,6 +1692,12 @@
 )</t>
         </is>
       </c>
+      <c r="J20" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K20" s="6" t="n">
+        <v>73.09999999999999</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -1620,6 +1744,12 @@
         <is>
           <t>df["JoinDate"] = df["JoinDate"].fillna(df["JoinDate"].mode()[0])</t>
         </is>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>69.2</v>
       </c>
     </row>
     <row r="22">
@@ -1670,6 +1800,12 @@
 ).dt.strftime("%Y-%m-%d")</t>
         </is>
       </c>
+      <c r="J22" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K22" s="6" t="n">
+        <v>69.2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -1717,6 +1853,12 @@
           <t>import numpy as np
 df["JoinDate"] = df["JoinDate"].replace("TBD", np.nan)</t>
         </is>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K23" s="6" t="n">
+        <v>69.2</v>
       </c>
     </row>
     <row r="24">
@@ -1767,6 +1909,12 @@
 )</t>
         </is>
       </c>
+      <c r="J24" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K24" s="6" t="n">
+        <v>69.2</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -1816,6 +1964,12 @@
 )</t>
         </is>
       </c>
+      <c r="J25" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K25" s="6" t="n">
+        <v>69.2</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -1862,6 +2016,12 @@
         <is>
           <t>df["AccountBalance"] = df["AccountBalance"].fillna(df["AccountBalance"].mode()[0])</t>
         </is>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K26" s="6" t="n">
+        <v>69.2</v>
       </c>
     </row>
     <row r="27">
@@ -1913,6 +2073,12 @@
 )</t>
         </is>
       </c>
+      <c r="J27" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K27" s="6" t="n">
+        <v>69.2</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -1962,6 +2128,12 @@
 )</t>
         </is>
       </c>
+      <c r="J28" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K28" s="6" t="n">
+        <v>69.2</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -2011,6 +2183,12 @@
 )</t>
         </is>
       </c>
+      <c r="J29" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K29" s="6" t="n">
+        <v>69.2</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -2058,6 +2236,12 @@
           <t>import numpy as np
 df["AccountBalance"] = df["AccountBalance"].replace("TBD", np.nan)</t>
         </is>
+      </c>
+      <c r="J30" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K30" s="6" t="n">
+        <v>69.2</v>
       </c>
     </row>
     <row r="31">
@@ -2108,6 +2292,12 @@
 )</t>
         </is>
       </c>
+      <c r="J31" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K31" s="6" t="n">
+        <v>69.2</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -2157,6 +2347,12 @@
 )</t>
         </is>
       </c>
+      <c r="J32" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K32" s="6" t="n">
+        <v>69.2</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -2203,6 +2399,12 @@
         <is>
           <t>df["Status"] = df["Status"].fillna(df["Status"].mode()[0])</t>
         </is>
+      </c>
+      <c r="J33" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K33" s="6" t="n">
+        <v>30.8</v>
       </c>
     </row>
     <row r="34">
@@ -2253,6 +2455,12 @@
 suspect = df.loc[mask, "Status"]</t>
         </is>
       </c>
+      <c r="J34" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K34" s="6" t="n">
+        <v>30.8</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -2300,6 +2508,12 @@
           <t>import numpy as np
 df["Status"] = df["Status"].replace("TBD", np.nan)</t>
         </is>
+      </c>
+      <c r="J35" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K35" s="6" t="n">
+        <v>30.8</v>
       </c>
     </row>
     <row r="36">
@@ -2350,6 +2564,12 @@
 )</t>
         </is>
       </c>
+      <c r="J36" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K36" s="6" t="n">
+        <v>30.8</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -2397,6 +2617,12 @@
           <t>df["ZipCode"] = df["ZipCode"].fillna(df["ZipCode"].mode()[0])</t>
         </is>
       </c>
+      <c r="J37" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K37" s="6" t="n">
+        <v>73.09999999999999</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -2445,6 +2671,12 @@
 df["ZipCode"] = df["ZipCode"].replace("00000", np.nan)</t>
         </is>
       </c>
+      <c r="J38" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K38" s="6" t="n">
+        <v>73.09999999999999</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -2492,6 +2724,12 @@
           <t>import numpy as np
 df["ZipCode"] = df["ZipCode"].replace("TBD", np.nan)</t>
         </is>
+      </c>
+      <c r="J39" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K39" s="6" t="n">
+        <v>73.09999999999999</v>
       </c>
     </row>
     <row r="40">
@@ -2542,6 +2780,12 @@
 )</t>
         </is>
       </c>
+      <c r="J40" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K40" s="6" t="n">
+        <v>73.09999999999999</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
@@ -2590,6 +2834,12 @@
     df["ZipCode"] == "12345"
 )</t>
         </is>
+      </c>
+      <c r="J41" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K41" s="6" t="n">
+        <v>73.09999999999999</v>
       </c>
     </row>
     <row r="42">
@@ -2641,6 +2891,12 @@
 df["Notes"] = df["Notes"].fillna("MISSING")</t>
         </is>
       </c>
+      <c r="J42" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="K42" s="6" t="n">
+        <v>73.3</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -2689,6 +2945,12 @@
 df["Notes"] = df["Notes"].replace("TEST", np.nan)</t>
         </is>
       </c>
+      <c r="J43" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="K43" s="6" t="n">
+        <v>73.3</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -2736,6 +2998,12 @@
           <t>import numpy as np
 df["Notes"] = df["Notes"].replace("TBD", np.nan)</t>
         </is>
+      </c>
+      <c r="J44" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="K44" s="6" t="n">
+        <v>73.3</v>
       </c>
     </row>
     <row r="45">
@@ -2785,6 +3053,12 @@
     df["Notes"] == "Preferred customer"
 )</t>
         </is>
+      </c>
+      <c r="J45" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="K45" s="6" t="n">
+        <v>73.3</v>
       </c>
     </row>
     <row r="46">
@@ -3082,6 +3356,12 @@
 ).dt.strftime("%Y-%m-%d")</t>
         </is>
       </c>
+      <c r="J51" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K51" s="6" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
@@ -3132,6 +3412,12 @@
 )</t>
         </is>
       </c>
+      <c r="J52" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K52" s="6" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
@@ -3178,6 +3464,12 @@
         <is>
           <t>df["ShipDate"] = df["ShipDate"].fillna(df["ShipDate"].mode()[0])</t>
         </is>
+      </c>
+      <c r="J53" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K53" s="6" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="54">
@@ -3228,6 +3520,12 @@
 ).dt.strftime("%Y-%m-%d")</t>
         </is>
       </c>
+      <c r="J54" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K54" s="6" t="n">
+        <v>75</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
@@ -3277,6 +3575,12 @@
 suspect = df.loc[mask, "Status"]</t>
         </is>
       </c>
+      <c r="J55" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K55" s="6" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
@@ -3326,6 +3630,12 @@
 suspect = df.loc[mask, "Status"]</t>
         </is>
       </c>
+      <c r="J56" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K56" s="6" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
@@ -3375,6 +3685,12 @@
 suspect = df.loc[mask, "Status"]</t>
         </is>
       </c>
+      <c r="J57" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K57" s="6" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
@@ -3422,6 +3738,12 @@
           <t>import numpy as np
 df["Status"] = df["Status"].replace("Test", np.nan)</t>
         </is>
+      </c>
+      <c r="J58" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K58" s="6" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="59">

</xml_diff>

<commit_message>
fix(score): soft-floor health score so catastrophic sheets read as "critical" not 0
Replace the hard max(0, ...) clamp in _compute_health_score with a soft-floor
transform: scores >= 25 are unchanged (raw 100-minus-penalties, preserving the
normal range and ranking exactly), while scores below 25 are compressed toward
an ~8 asymptote instead of saturating at 0. Strictly monotonic — worse data is
always a lower score. Penalty accumulation is untouched; only the final clamp
changed.

Add a "Critical" band to score_label (>=40 significant issues, else critical)
so single-digit scores read with a word.

Sample effect: Customers 0 -> 18, Orders 65 (unchanged), overall 32 -> 42.

Re-snapshot README CLI example and regenerate samples/output reports
(HTML/PDF/xlsx). Update tests: rename the floors-at-zero test to
never-negative and add a catastrophic-sheet test asserting single-digit floor
that never hits 0 or below.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/output/sample_messy_data_audit_findings.xlsx
+++ b/samples/output/sample_messy_data_audit_findings.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>32/100</t>
+          <t>42/100</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07 18:48:43</t>
+          <t>2026-07-08 15:09:34</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Score: 0/100</t>
+          <t>Score: 18/100</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: regenerate both sample report sets with 1.2.0 output
Refresh the committed messy (42/100) and realistic (67/100) HTML/Excel/PDF
deliverables so they reflect the unified issue wording, score-band, and
score-ring changes in 1.2.0. Scores and tallies unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/output/sample_messy_data_audit_findings.xlsx
+++ b/samples/output/sample_messy_data_audit_findings.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Findings'!$A$1:$I$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Findings'!$A$1:$K$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -540,7 +540,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15 09:02:00</t>
+          <t>2026-07-27 16:58:34</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>Mixed ID formats</t>
+          <t>Mixed ID formats: e.g. "29 coded (e.g. CUST-001) vs 1 bare numbers"</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>4 of 30 values missing (13.3%)</t>
+          <t>High missing rate: 4 of 30 values missing (13.3%)</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Code/ID stuffed in name field</t>
+          <t>Code/ID stuffed in name field: e.g. "REF-4421"</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Placeholder "Test" found 3 times</t>
+          <t>Placeholder: "Test" appears 3 times (11.5%)</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Placeholder "TBD" found 1 times</t>
+          <t>Placeholder: "TBD" appears 1 times (3.8%)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>4 of 30 values missing (13.3%)</t>
+          <t>High missing rate: 4 of 30 values missing (13.3%)</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Placeholder "TBD" found 1 times</t>
+          <t>Placeholder: "TBD" appears 1 times (3.8%)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>"User" repeated 3 times</t>
+          <t>Suspicious repetition: "User" appears 3 times (11.5%)</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>"Doe" repeated 3 times</t>
+          <t>Suspicious repetition: "Doe" appears 3 times (11.5%)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>4 of 30 values missing (13.3%)</t>
+          <t>High missing rate: 4 of 30 values missing (13.3%)</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Invalid email format</t>
+          <t>Invalid email format: e.g. "henrylee"</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Invalid email format</t>
+          <t>Invalid email format: e.g. "nancy w@example.com"</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>"test@test.com" repeated 3 times</t>
+          <t>Suspicious repetition: "test@test.com" appears 3 times (11.5%)</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>4 of 30 values missing (13.3%)</t>
+          <t>High missing rate: 4 of 30 values missing (13.3%)</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Mixed phone formats: 17 values deviate from (XXX) XXX-XXXX</t>
+          <t>Mixed phone formats: 17 of 26 values deviate from (XXX) XXX-XXXX</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Placeholder "TBD" found 1 times</t>
+          <t>Placeholder: "TBD" appears 1 times (3.8%)</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>"(555) 123-4567" repeated 3 times</t>
+          <t>Suspicious repetition: "(555) 123-4567" appears 3 times (11.5%)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>"000-000-0000" repeated 3 times</t>
+          <t>Suspicious repetition: "000-000-0000" appears 3 times (11.5%)</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>"555-555-5555" repeated 3 times</t>
+          <t>Suspicious repetition: "555-555-5555" appears 3 times (11.5%)</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>4 of 30 values missing (13.3%)</t>
+          <t>High missing rate: 4 of 30 values missing (13.3%)</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Mixed date formats: 12 values deviate from YYYY-MM-DD</t>
+          <t>Mixed date formats: 12 of 26 values deviate from YYYY-MM-DD</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Placeholder "TBD" found 1 times</t>
+          <t>Placeholder: "TBD" appears 1 times (3.8%)</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>"2023-01-01" repeated 6 times</t>
+          <t>Suspicious repetition: "2023-01-01" appears 6 times (23.1%)</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>"2023-01-15" repeated 3 times</t>
+          <t>Suspicious repetition: "2023-01-15" appears 3 times (11.5%)</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>4 of 30 values missing (13.3%)</t>
+          <t>High missing rate: 4 of 30 values missing (13.3%)</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -2052,7 +2052,7 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Mixed currency formats: 11 values deviate from $X,XXX.XX</t>
+          <t>Mixed currency formats: 11 of 26 values deviate from $X,XXX.XX</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>Text in currency field</t>
+          <t>Text in currency field: e.g. "TBD"</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>Text in currency field</t>
+          <t>Text in currency field: e.g. "five thousand"</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>Placeholder "TBD" found 1 times</t>
+          <t>Placeholder: "TBD" appears 1 times (3.8%)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>"$0.00" repeated 6 times</t>
+          <t>Suspicious repetition: "$0.00" appears 6 times (23.1%)</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>"$1,250.00" repeated 3 times</t>
+          <t>Suspicious repetition: "$1,250.00" appears 3 times (11.5%)</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>4 of 30 values missing (13.3%)</t>
+          <t>High missing rate: 4 of 30 values missing (13.3%)</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>Inconsistent casing in categorical values</t>
+          <t>Inconsistent casing in categorical values: e.g. "ACTIVE / Active / active"</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>Placeholder "TBD" found 1 times</t>
+          <t>Placeholder: "TBD" appears 1 times (3.8%)</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>"Active" repeated 18 times</t>
+          <t>Suspicious repetition: "Active" appears 18 times (69.2%)</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>4 of 30 values missing (13.3%)</t>
+          <t>High missing rate: 4 of 30 values missing (13.3%)</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>Placeholder "00000" found 3 times</t>
+          <t>Placeholder: "00000" appears 3 times (11.5%)</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>Placeholder "TBD" found 1 times</t>
+          <t>Placeholder: "TBD" appears 1 times (3.8%)</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>"30301" repeated 3 times</t>
+          <t>Suspicious repetition: "30301" appears 3 times (11.5%)</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>"12345" repeated 3 times</t>
+          <t>Suspicious repetition: "12345" appears 3 times (11.5%)</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>15 of 30 values missing (50.0%)</t>
+          <t>High missing rate: 15 of 30 values missing (50.0%)</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>Placeholder "TEST" found 3 times</t>
+          <t>Placeholder: "TEST" appears 3 times (20.0%)</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>Placeholder "TBD" found 1 times</t>
+          <t>Placeholder: "TBD" appears 1 times (6.7%)</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>"Preferred customer" repeated 3 times</t>
+          <t>Suspicious repetition: "Preferred customer" appears 3 times (20.0%)</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>Mixed date formats: 4 values deviate from YYYY-MM-DD</t>
+          <t>Mixed date formats: 4 of 10 values deviate from YYYY-MM-DD</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>Mixed currency formats: 3 values deviate from $X,XXX.XX</t>
+          <t>Mixed currency formats: 3 of 10 values deviate from $X,XXX.XX</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
@@ -3447,7 +3447,7 @@
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>2 of 10 values missing (20.0%)</t>
+          <t>High missing rate: 2 of 10 values missing (20.0%)</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
@@ -3500,7 +3500,7 @@
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>Mixed date formats: 3 values deviate from YYYY-MM-DD</t>
+          <t>Mixed date formats: 3 of 8 values deviate from YYYY-MM-DD</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>Inconsistent casing in categorical values</t>
+          <t>Inconsistent casing in categorical values: e.g. "Shipped / shipped"</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">
@@ -3610,7 +3610,7 @@
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>Inconsistent casing in categorical values</t>
+          <t>Inconsistent casing in categorical values: e.g. "Delivered / delivered"</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>Inconsistent casing in categorical values</t>
+          <t>Inconsistent casing in categorical values: e.g. "PENDING / Pending"</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>Placeholder "Test" found 2 times</t>
+          <t>Placeholder: "Test" appears 2 times (20.0%)</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
@@ -3841,7 +3841,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I60"/>
+  <autoFilter ref="A1:K60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(samples): regenerate showcase reports from 1.3.0 + fix README date-pattern count
Prompt 6 step 0.f. The committed samples/output/ reports were last regenerated
at 1.2.0; regenerate them from current source so the shipped showcase reflects
the 1.3.0 tool (visible counts unchanged — 59 issues 23H/20M/16L, health 42/100
— since they already footed). README "What It Detects" said 6 date patterns;
DATE_PATTERNS actually has 9 (phone 7 / currency 6 were correct).

Verified with engagement-template/scripts/scan_binaries_for_drift.py: 0 retired
tokens across all 6 tracked binaries (char counts confirm real extraction), the
scenario the 2026-08-04 binary scan named as most likely to reintroduce a figure.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/output/sample_messy_data_audit_findings.xlsx
+++ b/samples/output/sample_messy_data_audit_findings.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Findings" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Findings'!$A$1:$K$60</definedName>
@@ -540,7 +540,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27 16:58:34</t>
+          <t>2026-08-05 20:45:07</t>
         </is>
       </c>
     </row>

</xml_diff>